<commit_message>
feat: update bilingual gallery and responsive images
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rf446d2db101d4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R5aa06834c847436d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R922a9389c44b4476"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R4003608dfa154b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R9c5bfe8de9f34eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="Reb301f80e6e84935"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R5e275dce64764e59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="Rc6b306b142e74049"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R7a04cd2ad5f843a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rc1a106a8df0c4cb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R391d607e158d4fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R7dc5758150e84b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R48d448f6a1874802"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="Ra27ce088b7d34d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R088e75820ca74747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="Re4943b696a474e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="Rfca71930f7bf4b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R25b9f0d4ce644078"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1362,9 +1362,6 @@
     <x:t xml:space="preserve">gallery_001</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">济州松岳山日出</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20260515_%E6%B5%8E%E5%B7%9E%E6%9D%BE%E5%B2%B3%E5%B1%B1%E6%97%A5%E5%87%BA.webp</x:t>
   </x:si>
   <x:si>
@@ -1374,9 +1371,6 @@
     <x:t xml:space="preserve">gallery_002</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">大变蛋糕人</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20260329_%E5%A4%A7%E5%8F%98%E8%9B%8B%E7%B3%95%E4%BA%BA.webp</x:t>
   </x:si>
   <x:si>
@@ -1386,9 +1380,6 @@
     <x:t xml:space="preserve">gallery_003</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">济州卡丁车</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20260328_%E6%B5%8E%E5%B7%9E%E5%8D%A1%E4%B8%81%E8%BD%A6.webp</x:t>
   </x:si>
   <x:si>
@@ -1398,9 +1389,6 @@
     <x:t xml:space="preserve">gallery_004</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">马头人滑雪</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20260223_%E9%A9%AC%E5%A4%B4%E4%BA%BA%E6%BB%91%E9%9B%AA.webp</x:t>
   </x:si>
   <x:si>
@@ -1410,9 +1398,6 @@
     <x:t xml:space="preserve">gallery_005</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">智异山顶</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20260201_%E6%99%BA%E5%BC%82%E5%B1%B1%E9%A1%B6.webp</x:t>
   </x:si>
   <x:si>
@@ -1422,9 +1407,6 @@
     <x:t xml:space="preserve">gallery_006</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">BK+统营</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20260106_BK%2B%E7%BB%9F%E8%90%A5.webp</x:t>
   </x:si>
   <x:si>
@@ -1434,9 +1416,6 @@
     <x:t xml:space="preserve">gallery_007</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">大变圣诞老人</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20251126_%E5%A4%A7%E5%8F%98%E5%9C%A3%E8%AF%9E%E8%80%81%E4%BA%BA.webp</x:t>
   </x:si>
   <x:si>
@@ -1446,9 +1425,6 @@
     <x:t xml:space="preserve">gallery_008</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">釜山烟花节</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20251115_%E9%87%9C%E5%B1%B1%E7%83%9F%E8%8A%B1%E8%8A%82.webp</x:t>
   </x:si>
   <x:si>
@@ -1458,9 +1434,6 @@
     <x:t xml:space="preserve">gallery_009</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">温哥华SENSORS</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20251027_%E6%B8%A9%E5%93%A5%E5%8D%8ESENSORS.webp</x:t>
   </x:si>
   <x:si>
@@ -1470,9 +1443,6 @@
     <x:t xml:space="preserve">gallery_010</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">米菲70周年</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20251007_%E7%B1%B3%E8%8F%B270%E5%91%A8%E5%B9%B4.webp</x:t>
   </x:si>
   <x:si>
@@ -1482,9 +1452,6 @@
     <x:t xml:space="preserve">gallery_011</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">丽水楠哥婚礼</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20251002_%E4%B8%BD%E6%B0%B4%E6%A5%A0%E5%93%A5%E5%A9%9A%E7%A4%BC.webp</x:t>
   </x:si>
   <x:si>
@@ -1494,9 +1461,6 @@
     <x:t xml:space="preserve">gallery_012</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">MNTL谭阳</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250828_MNTL%E8%B0%AD%E9%98%B3.webp</x:t>
   </x:si>
   <x:si>
@@ -1506,9 +1470,6 @@
     <x:t xml:space="preserve">gallery_013</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">BK FellowShip 奖学金</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250826_BK%20FellowShip%20%E5%A5%96%E5%AD%A6%E9%87%91.webp</x:t>
   </x:si>
   <x:si>
@@ -1518,9 +1479,6 @@
     <x:t xml:space="preserve">gallery_014</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Dr.Nomin</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250524_Dr.Nomin.webp</x:t>
   </x:si>
   <x:si>
@@ -1530,9 +1488,6 @@
     <x:t xml:space="preserve">gallery_015</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">浦项SpaceWalk</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250504_%E6%B5%A6%E9%A1%B9SpaceWalk.webp</x:t>
   </x:si>
   <x:si>
@@ -1542,9 +1497,6 @@
     <x:t xml:space="preserve">gallery_016</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">济州枪击</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250328_%E6%B5%8E%E5%B7%9E%E6%9E%AA%E5%87%BB.webp</x:t>
   </x:si>
   <x:si>
@@ -1554,9 +1506,6 @@
     <x:t xml:space="preserve">gallery_017</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">羽毛球比赛</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250309_%E7%BE%BD%E6%AF%9B%E7%90%83%E6%AF%94%E8%B5%9B.webp</x:t>
   </x:si>
   <x:si>
@@ -1566,9 +1515,6 @@
     <x:t xml:space="preserve">gallery_018</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">RLRC最佳研究生</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250227_RLRC%E6%9C%80%E4%BD%B3%E7%A0%94%E7%A9%B6%E7%94%9F.webp</x:t>
   </x:si>
   <x:si>
@@ -1578,9 +1524,6 @@
     <x:t xml:space="preserve">gallery_019</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">福州添福</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250204_%E7%A6%8F%E5%B7%9E%E6%B7%BB%E7%A6%8F.webp</x:t>
   </x:si>
   <x:si>
@@ -1590,9 +1533,6 @@
     <x:t xml:space="preserve">gallery_020</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">大变财神</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250202_%E5%A4%A7%E5%8F%98%E8%B4%A2%E7%A5%9E.webp</x:t>
   </x:si>
   <x:si>
@@ -1602,9 +1542,6 @@
     <x:t xml:space="preserve">gallery_021</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">杭州径山</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20250129_%E6%9D%AD%E5%B7%9E%E5%BE%84%E5%B1%B1.webp</x:t>
   </x:si>
   <x:si>
@@ -1614,9 +1551,6 @@
     <x:t xml:space="preserve">gallery_022</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">圣诞节+汉拿山</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20241225_%E5%9C%A3%E8%AF%9E%E8%8A%82%2B%E6%B1%89%E6%8B%BF%E5%B1%B1.webp</x:t>
   </x:si>
   <x:si>
@@ -1626,9 +1560,6 @@
     <x:t xml:space="preserve">gallery_023</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">釜山海上烟花</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20241122_%E9%87%9C%E5%B1%B1%E6%B5%B7%E4%B8%8A%E7%83%9F%E8%8A%B1.webp</x:t>
   </x:si>
   <x:si>
@@ -1638,9 +1569,6 @@
     <x:t xml:space="preserve">gallery_024</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">无等山顶</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20241116_%E6%97%A0%E7%AD%89%E5%B1%B1%E9%A1%B6.webp</x:t>
   </x:si>
   <x:si>
@@ -1650,9 +1578,6 @@
     <x:t xml:space="preserve">gallery_025</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">釜山海云台</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20240803_%E9%87%9C%E5%B1%B1%E6%B5%B7%E4%BA%91%E5%8F%B0.webp</x:t>
   </x:si>
   <x:si>
@@ -1662,9 +1587,6 @@
     <x:t xml:space="preserve">gallery_026</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">动物园</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20240410_%E5%8A%A8%E7%89%A9%E5%9B%AD.webp</x:t>
   </x:si>
   <x:si>
@@ -1674,9 +1596,6 @@
     <x:t xml:space="preserve">gallery_027</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">济州汉拿山</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20240316_%E6%B5%8E%E5%B7%9E%E6%B1%89%E6%8B%BF%E5%B1%B1.webp</x:t>
   </x:si>
   <x:si>
@@ -1686,9 +1605,6 @@
     <x:t xml:space="preserve">gallery_028</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">茂朱滑雪</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20240124_%E8%8C%82%E6%9C%B1%E6%BB%91%E9%9B%AA.webp</x:t>
   </x:si>
   <x:si>
@@ -1698,9 +1614,6 @@
     <x:t xml:space="preserve">gallery_029</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">我和雪人</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20231216_%E6%88%91%E5%92%8C%E9%9B%AA%E4%BA%BA.webp</x:t>
   </x:si>
   <x:si>
@@ -1710,9 +1623,6 @@
     <x:t xml:space="preserve">gallery_030</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">波兰卡托维兹μTAS</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20231019_%E6%B3%A2%E5%85%B0%E5%8D%A1%E6%89%98%E7%BB%B4%E5%85%B9%CE%BCTAS.webp</x:t>
   </x:si>
   <x:si>
@@ -1722,9 +1632,6 @@
     <x:t xml:space="preserve">gallery_031</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">釜山广安里</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20230823_%E9%87%9C%E5%B1%B1%E5%B9%BF%E5%AE%89%E9%87%8C.webp</x:t>
   </x:si>
   <x:si>
@@ -1734,9 +1641,6 @@
     <x:t xml:space="preserve">gallery_032</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">济州牛岛</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20230730_%E6%B5%8E%E5%B7%9E%E7%89%9B%E5%B2%9B.webp</x:t>
   </x:si>
   <x:si>
@@ -1746,9 +1650,6 @@
     <x:t xml:space="preserve">gallery_033</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Dr. Dongsu 婚礼</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20230513_Dr.%20Dongsu%E5%A9%9A%E7%A4%BC.webp</x:t>
   </x:si>
   <x:si>
@@ -1758,9 +1659,6 @@
     <x:t xml:space="preserve">gallery_034</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">过年</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20230121_%E8%BF%87%E5%B9%B4.webp</x:t>
   </x:si>
   <x:si>
@@ -1770,9 +1668,6 @@
     <x:t xml:space="preserve">gallery_035</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">光州无等山</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20221119_%E5%85%89%E5%B7%9E%E6%97%A0%E7%AD%89%E5%B1%B1.webp</x:t>
   </x:si>
   <x:si>
@@ -1780,9 +1675,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">gallery_036</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">抵达韩国</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">assets/albums-optimized/20220901_%E6%8A%B5%E8%BE%BE%E9%9F%A9%E5%9B%BD.webp</x:t>
@@ -2392,8 +2284,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -2493,7 +2386,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2552,6 +2445,7 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -2701,8 +2595,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J37">
-  <x:autoFilter ref="A1:J37"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J42" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J42"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="date"/>
@@ -3095,7 +2989,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fc45dd97a945c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2df0ca8d5a25459e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3708,7 +3602,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e748b5833f8407c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4d48cb48bc14033"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4363,7 +4257,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R331adee6c5cc44a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2092621003fb4748"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4769,7 +4663,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea321d716e524f3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f8dcf4ea3aa40ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5173,7 +5067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b82a1b394a04ce0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a73f7bec4fe44a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5412,7 +5306,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c4f70e2ceed46e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e0c81c7a9a0428c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5470,862 +5364,982 @@
       <x:c r="B2" s="12">
         <x:v>46157</x:v>
       </x:c>
-      <x:c r="C2" s="4" t="s">
+      <x:c r="C2" s="4" t="str">
+        <x:v>Sunrise at Songaksan, Jeju</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="str">
+        <x:v>济州松岳山日出</x:v>
+      </x:c>
+      <x:c r="E2" s="4" t="s">
         <x:v>423</x:v>
-      </x:c>
-      <x:c r="D2" s="4" t="s">
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="s">
-        <x:v>424</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4" t="s">
-        <x:v>425</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="J2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="11" t="s">
-        <x:v>426</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="B3" s="13">
         <x:v>46110</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="s">
-        <x:v>427</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="s">
-        <x:v>427</x:v>
+      <x:c r="C3" s="5" t="str">
+        <x:v>Become Cake Man</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="str">
+        <x:v>大变蛋糕人</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>428</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="F3" s="5"/>
       <x:c r="G3" s="5"/>
       <x:c r="H3" s="5"/>
       <x:c r="I3" s="5" t="s">
-        <x:v>429</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="J3" s="7"/>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="11" t="s">
-        <x:v>430</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="B4" s="13">
         <x:v>46109</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
-        <x:v>431</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>431</x:v>
+      <x:c r="C4" s="5" t="str">
+        <x:v>Go-Karting in Jeju</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="str">
+        <x:v>济州卡丁车</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>432</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="F4" s="5"/>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5" t="s">
-        <x:v>433</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="J4" s="7"/>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>434</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="B5" s="13">
         <x:v>46076</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="s">
-        <x:v>435</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="s">
-        <x:v>435</x:v>
+      <x:c r="C5" s="5" t="str">
+        <x:v>Horse-man Skiing</x:v>
+      </x:c>
+      <x:c r="D5" s="5" t="str">
+        <x:v>马头人滑雪</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>436</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="J5" s="7"/>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="B6" s="13">
         <x:v>46054</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>439</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>439</x:v>
+      <x:c r="C6" s="5" t="str">
+        <x:v>Summit of Jirisan</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="str">
+        <x:v>智异山顶</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>440</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5" t="s">
-        <x:v>441</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="J6" s="7"/>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>442</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="B7" s="13">
         <x:v>46028</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="s">
-        <x:v>443</x:v>
+      <x:c r="C7" s="5" t="str">
+        <x:v>BK Trip to Tongyeong</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="str">
+        <x:v>BK+统营</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>444</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="F7" s="5"/>
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5" t="s">
-        <x:v>445</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J7" s="7"/>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>446</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="B8" s="13">
         <x:v>45987</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>447</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>447</x:v>
+      <x:c r="C8" s="5" t="str">
+        <x:v>Become Santa Claus</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="str">
+        <x:v>大变圣诞老人</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>448</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="F8" s="5"/>
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5" t="s">
-        <x:v>449</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="J8" s="7"/>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>450</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="B9" s="13">
         <x:v>45976</x:v>
       </x:c>
-      <x:c r="C9" s="5" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
-        <x:v>451</x:v>
+      <x:c r="C9" s="5" t="str">
+        <x:v>Busan Fireworks Festival</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="str">
+        <x:v>釜山烟花节</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>452</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="F9" s="5"/>
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5" t="s">
-        <x:v>453</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="J9" s="7"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>454</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="B10" s="13">
         <x:v>45957</x:v>
       </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>455</x:v>
+      <x:c r="C10" s="5" t="str">
+        <x:v>IEEE SENSORS 2025 in Vancouver</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="str">
+        <x:v>温哥华SENSORS</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>456</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="F10" s="5"/>
       <x:c r="G10" s="5"/>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5" t="s">
-        <x:v>457</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="J10" s="7"/>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>458</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="B11" s="13">
         <x:v>45937</x:v>
       </x:c>
-      <x:c r="C11" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="s">
-        <x:v>459</x:v>
+      <x:c r="C11" s="5" t="str">
+        <x:v>Miffy 70th Anniversary</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="str">
+        <x:v>米菲70周年</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="F11" s="5"/>
       <x:c r="G11" s="5"/>
       <x:c r="H11" s="5"/>
       <x:c r="I11" s="5" t="s">
-        <x:v>461</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="J11" s="7"/>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>462</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B12" s="13">
         <x:v>45932</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>463</x:v>
+      <x:c r="C12" s="5" t="str">
+        <x:v>Nan's Wedding</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="str">
+        <x:v>丽水楠哥婚礼</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="F12" s="5"/>
       <x:c r="G12" s="5"/>
       <x:c r="H12" s="5"/>
       <x:c r="I12" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="J12" s="7"/>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="11" t="s">
-        <x:v>466</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="B13" s="13">
         <x:v>45897</x:v>
       </x:c>
-      <x:c r="C13" s="5" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="D13" s="5" t="s">
-        <x:v>467</x:v>
+      <x:c r="C13" s="5" t="str">
+        <x:v>MNTL workshop to Damyang</x:v>
+      </x:c>
+      <x:c r="D13" s="5" t="str">
+        <x:v>MNTL谭阳</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="F13" s="5"/>
       <x:c r="G13" s="5"/>
       <x:c r="H13" s="5"/>
       <x:c r="I13" s="5" t="s">
-        <x:v>469</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="J13" s="7"/>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="11" t="s">
-        <x:v>470</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B14" s="13">
         <x:v>45895</x:v>
       </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>471</x:v>
+      <x:c r="C14" s="5" t="str">
+        <x:v>BK21 Fellowship Scholarship</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="str">
+        <x:v>BK FellowShip 奖学金</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>472</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F14" s="5"/>
       <x:c r="G14" s="5"/>
       <x:c r="H14" s="5"/>
       <x:c r="I14" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="J14" s="7"/>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="11" t="s">
-        <x:v>474</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="B15" s="13">
         <x:v>45801</x:v>
       </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="D15" s="5" t="s">
-        <x:v>475</x:v>
+      <x:c r="C15" s="5" t="str">
+        <x:v>Dinner with Dr. Nomin</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="str">
+        <x:v>Dr.Nomin 聚餐</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>476</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="F15" s="5"/>
       <x:c r="G15" s="5"/>
       <x:c r="H15" s="5"/>
       <x:c r="I15" s="5" t="s">
-        <x:v>477</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="J15" s="7"/>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>478</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B16" s="13">
         <x:v>45781</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>479</x:v>
-      </x:c>
-      <x:c r="D16" s="5" t="s">
-        <x:v>479</x:v>
+      <x:c r="C16" s="5" t="str">
+        <x:v>Space Walk in Pohang</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="str">
+        <x:v>浦项SpaceWalk</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>480</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="5"/>
       <x:c r="I16" s="5" t="s">
-        <x:v>481</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="J16" s="7"/>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="11" t="s">
-        <x:v>482</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B17" s="13">
         <x:v>45744</x:v>
       </x:c>
-      <x:c r="C17" s="5" t="s">
-        <x:v>483</x:v>
-      </x:c>
-      <x:c r="D17" s="5" t="s">
-        <x:v>483</x:v>
+      <x:c r="C17" s="5" t="str">
+        <x:v>Shooting in Jeju</x:v>
+      </x:c>
+      <x:c r="D17" s="5" t="str">
+        <x:v>济州枪击</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>484</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="F17" s="5"/>
       <x:c r="G17" s="5"/>
       <x:c r="H17" s="5"/>
       <x:c r="I17" s="5" t="s">
-        <x:v>485</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="J17" s="7"/>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>486</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="B18" s="13">
         <x:v>45725</x:v>
       </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>487</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="s">
-        <x:v>487</x:v>
+      <x:c r="C18" s="5" t="str">
+        <x:v>Badminton Tournament</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="str">
+        <x:v>羽毛球比赛</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="F18" s="5"/>
       <x:c r="G18" s="5"/>
       <x:c r="H18" s="5"/>
       <x:c r="I18" s="5" t="s">
-        <x:v>489</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="J18" s="7"/>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="11" t="s">
-        <x:v>490</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B19" s="13">
         <x:v>45715</x:v>
       </x:c>
-      <x:c r="C19" s="5" t="s">
-        <x:v>491</x:v>
-      </x:c>
-      <x:c r="D19" s="5" t="s">
-        <x:v>491</x:v>
+      <x:c r="C19" s="5" t="str">
+        <x:v>RLRC Outstanding Graduate Student</x:v>
+      </x:c>
+      <x:c r="D19" s="5" t="str">
+        <x:v>RLRC最佳研究生</x:v>
       </x:c>
       <x:c r="E19" s="5" t="s">
-        <x:v>492</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
       <x:c r="H19" s="5"/>
       <x:c r="I19" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="J19" s="7"/>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="11" t="s">
-        <x:v>494</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="B20" s="13">
         <x:v>45692</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>495</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>495</x:v>
+      <x:c r="C20" s="5" t="str">
+        <x:v>Travel in Fuzhou</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="str">
+        <x:v>福州添福</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>496</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="F20" s="5"/>
       <x:c r="G20" s="5"/>
       <x:c r="H20" s="5"/>
       <x:c r="I20" s="5" t="s">
-        <x:v>497</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="J20" s="7"/>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="11" t="s">
-        <x:v>498</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B21" s="13">
         <x:v>45690</x:v>
       </x:c>
-      <x:c r="C21" s="5" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="D21" s="5" t="s">
-        <x:v>499</x:v>
+      <x:c r="C21" s="5" t="str">
+        <x:v>Become God of Wealth</x:v>
+      </x:c>
+      <x:c r="D21" s="5" t="str">
+        <x:v>大变财神</x:v>
       </x:c>
       <x:c r="E21" s="5" t="s">
-        <x:v>500</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="F21" s="5"/>
       <x:c r="G21" s="5"/>
       <x:c r="H21" s="5"/>
       <x:c r="I21" s="5" t="s">
-        <x:v>501</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="J21" s="7"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="11" t="s">
-        <x:v>502</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B22" s="13">
         <x:v>45686</x:v>
       </x:c>
-      <x:c r="C22" s="5" t="s">
-        <x:v>503</x:v>
-      </x:c>
-      <x:c r="D22" s="5" t="s">
-        <x:v>503</x:v>
+      <x:c r="C22" s="5" t="str">
+        <x:v>Jingshan, Hangzhou</x:v>
+      </x:c>
+      <x:c r="D22" s="5" t="str">
+        <x:v>杭州径山</x:v>
       </x:c>
       <x:c r="E22" s="5" t="s">
-        <x:v>504</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="F22" s="5"/>
       <x:c r="G22" s="5"/>
       <x:c r="H22" s="5"/>
       <x:c r="I22" s="5" t="s">
-        <x:v>505</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="J22" s="7"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="11" t="s">
-        <x:v>506</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="B23" s="13">
         <x:v>45651</x:v>
       </x:c>
-      <x:c r="C23" s="5" t="s">
-        <x:v>507</x:v>
-      </x:c>
-      <x:c r="D23" s="5" t="s">
-        <x:v>507</x:v>
+      <x:c r="C23" s="5" t="str">
+        <x:v>Christmas at Summit of Hallasan</x:v>
+      </x:c>
+      <x:c r="D23" s="5" t="str">
+        <x:v>圣诞节+汉拿山</x:v>
       </x:c>
       <x:c r="E23" s="5" t="s">
-        <x:v>508</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="F23" s="5"/>
       <x:c r="G23" s="5"/>
       <x:c r="H23" s="5"/>
       <x:c r="I23" s="5" t="s">
-        <x:v>509</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="J23" s="7"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="11" t="s">
-        <x:v>510</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="B24" s="13">
         <x:v>45618</x:v>
       </x:c>
-      <x:c r="C24" s="5" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
-        <x:v>511</x:v>
+      <x:c r="C24" s="5" t="str">
+        <x:v>Fireworks over the Sea in Busan</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="str">
+        <x:v>釜山海上烟花</x:v>
       </x:c>
       <x:c r="E24" s="5" t="s">
-        <x:v>512</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="F24" s="5"/>
       <x:c r="G24" s="5"/>
       <x:c r="H24" s="5"/>
       <x:c r="I24" s="5" t="s">
-        <x:v>513</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="J24" s="7"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="11" t="s">
-        <x:v>514</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B25" s="13">
         <x:v>45612</x:v>
       </x:c>
-      <x:c r="C25" s="5" t="s">
-        <x:v>515</x:v>
-      </x:c>
-      <x:c r="D25" s="5" t="s">
-        <x:v>515</x:v>
+      <x:c r="C25" s="5" t="str">
+        <x:v>Summit of Mudeungsan</x:v>
+      </x:c>
+      <x:c r="D25" s="5" t="str">
+        <x:v>无等山顶</x:v>
       </x:c>
       <x:c r="E25" s="5" t="s">
-        <x:v>516</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F25" s="5"/>
       <x:c r="G25" s="5"/>
       <x:c r="H25" s="5"/>
       <x:c r="I25" s="5" t="s">
-        <x:v>517</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="J25" s="7"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="11" t="s">
-        <x:v>518</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="B26" s="13">
         <x:v>45507</x:v>
       </x:c>
-      <x:c r="C26" s="5" t="s">
-        <x:v>519</x:v>
-      </x:c>
-      <x:c r="D26" s="5" t="s">
-        <x:v>519</x:v>
+      <x:c r="C26" s="5" t="str">
+        <x:v>Haeundae, Busan</x:v>
+      </x:c>
+      <x:c r="D26" s="5" t="str">
+        <x:v>釜山海云台</x:v>
       </x:c>
       <x:c r="E26" s="5" t="s">
-        <x:v>520</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="F26" s="5"/>
       <x:c r="G26" s="5"/>
       <x:c r="H26" s="5"/>
       <x:c r="I26" s="5" t="s">
-        <x:v>521</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="J26" s="7"/>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="11" t="s">
-        <x:v>522</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B27" s="13">
         <x:v>45392</x:v>
       </x:c>
-      <x:c r="C27" s="5" t="s">
-        <x:v>523</x:v>
-      </x:c>
-      <x:c r="D27" s="5" t="s">
-        <x:v>523</x:v>
+      <x:c r="C27" s="5" t="str">
+        <x:v>Gwangju Zoo</x:v>
+      </x:c>
+      <x:c r="D27" s="5" t="str">
+        <x:v>动物园</x:v>
       </x:c>
       <x:c r="E27" s="5" t="s">
-        <x:v>524</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="F27" s="5"/>
       <x:c r="G27" s="5"/>
       <x:c r="H27" s="5"/>
       <x:c r="I27" s="5" t="s">
-        <x:v>525</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="J27" s="7"/>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="11" t="s">
-        <x:v>526</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B28" s="13">
         <x:v>45367</x:v>
       </x:c>
-      <x:c r="C28" s="5" t="s">
-        <x:v>527</x:v>
-      </x:c>
-      <x:c r="D28" s="5" t="s">
-        <x:v>527</x:v>
+      <x:c r="C28" s="5" t="str">
+        <x:v>1st Hallasan, Jeju</x:v>
+      </x:c>
+      <x:c r="D28" s="5" t="str">
+        <x:v>济州汉拿山</x:v>
       </x:c>
       <x:c r="E28" s="5" t="s">
-        <x:v>528</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="F28" s="5"/>
       <x:c r="G28" s="5"/>
       <x:c r="H28" s="5"/>
       <x:c r="I28" s="5" t="s">
-        <x:v>529</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="J28" s="7"/>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="11" t="s">
-        <x:v>530</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B29" s="13">
         <x:v>45315</x:v>
       </x:c>
-      <x:c r="C29" s="5" t="s">
-        <x:v>531</x:v>
-      </x:c>
-      <x:c r="D29" s="5" t="s">
-        <x:v>531</x:v>
+      <x:c r="C29" s="5" t="str">
+        <x:v>Skiing in Muju</x:v>
+      </x:c>
+      <x:c r="D29" s="5" t="str">
+        <x:v>茂朱滑雪</x:v>
       </x:c>
       <x:c r="E29" s="5" t="s">
-        <x:v>532</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="F29" s="5"/>
       <x:c r="G29" s="5"/>
       <x:c r="H29" s="5"/>
       <x:c r="I29" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="J29" s="7"/>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="11" t="s">
-        <x:v>534</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="B30" s="13">
         <x:v>45276</x:v>
       </x:c>
-      <x:c r="C30" s="5" t="s">
-        <x:v>535</x:v>
-      </x:c>
-      <x:c r="D30" s="5" t="s">
-        <x:v>535</x:v>
+      <x:c r="C30" s="5" t="str">
+        <x:v>Me and my Snowman</x:v>
+      </x:c>
+      <x:c r="D30" s="5" t="str">
+        <x:v>我和雪人</x:v>
       </x:c>
       <x:c r="E30" s="5" t="s">
-        <x:v>536</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="F30" s="5"/>
       <x:c r="G30" s="5"/>
       <x:c r="H30" s="5"/>
       <x:c r="I30" s="5" t="s">
-        <x:v>537</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="J30" s="7"/>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="11" t="s">
-        <x:v>538</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B31" s="13">
         <x:v>45218</x:v>
       </x:c>
-      <x:c r="C31" s="5" t="s">
-        <x:v>539</x:v>
-      </x:c>
-      <x:c r="D31" s="5" t="s">
-        <x:v>539</x:v>
+      <x:c r="C31" s="5" t="str">
+        <x:v>μTAS 2023 in Katowice, Poland</x:v>
+      </x:c>
+      <x:c r="D31" s="5" t="str">
+        <x:v>波兰卡托维兹μTAS</x:v>
       </x:c>
       <x:c r="E31" s="5" t="s">
-        <x:v>540</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="F31" s="5"/>
       <x:c r="G31" s="5"/>
       <x:c r="H31" s="5"/>
       <x:c r="I31" s="5" t="s">
-        <x:v>541</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="J31" s="7"/>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="11" t="s">
-        <x:v>542</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="B32" s="13">
         <x:v>45161</x:v>
       </x:c>
-      <x:c r="C32" s="5" t="s">
-        <x:v>543</x:v>
-      </x:c>
-      <x:c r="D32" s="5" t="s">
-        <x:v>543</x:v>
+      <x:c r="C32" s="5" t="str">
+        <x:v>Gwangalli, Busan</x:v>
+      </x:c>
+      <x:c r="D32" s="5" t="str">
+        <x:v>釜山广安里</x:v>
       </x:c>
       <x:c r="E32" s="5" t="s">
-        <x:v>544</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="F32" s="5"/>
       <x:c r="G32" s="5"/>
       <x:c r="H32" s="5"/>
       <x:c r="I32" s="5" t="s">
-        <x:v>545</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="J32" s="7"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="11" t="s">
-        <x:v>546</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B33" s="13">
         <x:v>45137</x:v>
       </x:c>
-      <x:c r="C33" s="5" t="s">
-        <x:v>547</x:v>
-      </x:c>
-      <x:c r="D33" s="5" t="s">
-        <x:v>547</x:v>
+      <x:c r="C33" s="5" t="str">
+        <x:v>Udo Island, Jeju</x:v>
+      </x:c>
+      <x:c r="D33" s="5" t="str">
+        <x:v>济州牛岛</x:v>
       </x:c>
       <x:c r="E33" s="5" t="s">
-        <x:v>548</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="F33" s="5"/>
       <x:c r="G33" s="5"/>
       <x:c r="H33" s="5"/>
       <x:c r="I33" s="5" t="s">
-        <x:v>549</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="J33" s="7"/>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="11" t="s">
-        <x:v>550</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="B34" s="13">
         <x:v>45059</x:v>
       </x:c>
-      <x:c r="C34" s="5" t="s">
-        <x:v>551</x:v>
-      </x:c>
-      <x:c r="D34" s="5" t="s">
-        <x:v>551</x:v>
+      <x:c r="C34" s="5" t="str">
+        <x:v>Dr. Dongsu's Wedding</x:v>
+      </x:c>
+      <x:c r="D34" s="5" t="str">
+        <x:v>Dr. Dongsu 婚礼</x:v>
       </x:c>
       <x:c r="E34" s="5" t="s">
-        <x:v>552</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="F34" s="5"/>
       <x:c r="G34" s="5"/>
       <x:c r="H34" s="5"/>
       <x:c r="I34" s="5" t="s">
-        <x:v>553</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="J34" s="7"/>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="11" t="s">
-        <x:v>554</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="B35" s="13">
         <x:v>44947</x:v>
       </x:c>
-      <x:c r="C35" s="5" t="s">
-        <x:v>555</x:v>
-      </x:c>
-      <x:c r="D35" s="5" t="s">
-        <x:v>555</x:v>
+      <x:c r="C35" s="5" t="str">
+        <x:v>Lunar New Year in Korea</x:v>
+      </x:c>
+      <x:c r="D35" s="5" t="str">
+        <x:v>韩国过年</x:v>
       </x:c>
       <x:c r="E35" s="5" t="s">
-        <x:v>556</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="F35" s="5"/>
       <x:c r="G35" s="5"/>
       <x:c r="H35" s="5"/>
       <x:c r="I35" s="5" t="s">
-        <x:v>557</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="J35" s="7"/>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="11" t="s">
-        <x:v>558</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="B36" s="13">
         <x:v>44884</x:v>
       </x:c>
-      <x:c r="C36" s="5" t="s">
-        <x:v>559</x:v>
-      </x:c>
-      <x:c r="D36" s="5" t="s">
-        <x:v>559</x:v>
+      <x:c r="C36" s="5" t="str">
+        <x:v>1st Mudeungsan, Gwangju</x:v>
+      </x:c>
+      <x:c r="D36" s="5" t="str">
+        <x:v>光州无等山</x:v>
       </x:c>
       <x:c r="E36" s="5" t="s">
-        <x:v>560</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="F36" s="5"/>
       <x:c r="G36" s="5"/>
       <x:c r="H36" s="5"/>
       <x:c r="I36" s="5" t="s">
-        <x:v>561</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="J36" s="7"/>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="11" t="s">
-        <x:v>562</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="B37" s="13">
         <x:v>44805</x:v>
       </x:c>
-      <x:c r="C37" s="5" t="s">
-        <x:v>563</x:v>
-      </x:c>
-      <x:c r="D37" s="5" t="s">
-        <x:v>563</x:v>
+      <x:c r="C37" s="5" t="str">
+        <x:v>Arrival in South Korea</x:v>
+      </x:c>
+      <x:c r="D37" s="5" t="str">
+        <x:v>抵达韩国</x:v>
       </x:c>
       <x:c r="E37" s="5" t="s">
-        <x:v>564</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="F37" s="5"/>
       <x:c r="G37" s="5"/>
       <x:c r="H37" s="5"/>
       <x:c r="I37" s="5" t="s">
-        <x:v>565</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="J37" s="7"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>gallery_037</x:v>
+      </x:c>
+      <x:c r="B38" s="17" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>Badminton Doubles Quarterfinals</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>羽毛球双打八强</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>assets/albums-optimized/20260711_%E7%BE%BD%E6%AF%9B%E7%90%83%E5%8F%8C%E6%89%93%E5%85%AB%E5%BC%BA.webp</x:v>
+      </x:c>
+      <x:c r="F38"/>
+      <x:c r="G38"/>
+      <x:c r="H38"/>
+      <x:c r="I38" t="str">
+        <x:v>20260711_羽毛球双打八强.jpg</x:v>
+      </x:c>
+      <x:c r="J38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>gallery_038</x:v>
+      </x:c>
+      <x:c r="B39" s="17" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>Jangheung Water Festival</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>长兴水庆典</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>assets/albums-optimized/20260730_%E9%95%BF%E5%85%B4%E6%B0%B4%E5%BA%86%E5%85%B8.webp</x:v>
+      </x:c>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+      <x:c r="I39" t="str">
+        <x:v>20260730_长兴水庆典.jpg</x:v>
+      </x:c>
+      <x:c r="J39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>gallery_039</x:v>
+      </x:c>
+      <x:c r="B40" s="17" t="n">
+        <x:v>46243</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>Car Accident in Jeju</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>济州撞车</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>assets/albums-optimized/20260809_%E6%B5%8E%E5%B7%9E%E6%92%9E%E8%BD%A6.webp</x:v>
+      </x:c>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+      <x:c r="I40" t="str">
+        <x:v>20260809_济州撞车.jpg</x:v>
+      </x:c>
+      <x:c r="J40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>gallery_040</x:v>
+      </x:c>
+      <x:c r="B41" s="17" t="n">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>"Fishing" at the Aquarium</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>水族馆"钓鱼"</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>assets/albums-optimized/20260810_%E6%B0%B4%E6%97%8F%E9%A6%86%E9%92%93%E9%B1%BC.webp</x:v>
+      </x:c>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+      <x:c r="I41" t="str">
+        <x:v>20260810_水族馆钓鱼.jpg</x:v>
+      </x:c>
+      <x:c r="J41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>gallery_041</x:v>
+      </x:c>
+      <x:c r="B42" s="17" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Damyang Bamboo Forest</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>谭阳竹林</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>assets/albums-optimized/20260907_%E8%B0%AD%E9%98%B3%E7%AB%B9%E6%9E%97.webp</x:v>
+      </x:c>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+      <x:c r="I42" t="str">
+        <x:v>20260907_谭阳竹林.jpg</x:v>
+      </x:c>
+      <x:c r="J42"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -6335,7 +6349,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9390b438fdc469a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61b6a7d90cdc4a7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6356,13 +6370,13 @@
   <x:sheetData>
     <x:row r="1" ht="27.950000762939453" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>566</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="B1" s="9" t="s">
-        <x:v>567</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>568</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
         <x:v>36</x:v>
@@ -6388,17 +6402,17 @@
     </x:row>
     <x:row r="2" ht="63.95000076293945" customHeight="1">
       <x:c r="A2" s="4" t="s">
-        <x:v>569</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="B2" s="10" t="s">
-        <x:v>570</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="C2" s="4"/>
       <x:c r="D2" s="4" t="s">
-        <x:v>571</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
-        <x:v>572</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4" t="s">
@@ -6414,19 +6428,19 @@
     </x:row>
     <x:row r="3" ht="63.95000076293945" customHeight="1">
       <x:c r="A3" s="5" t="s">
-        <x:v>573</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B3" s="11" t="s">
-        <x:v>574</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>575</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="D3" s="5" t="s">
-        <x:v>576</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>577</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="F3" s="5"/>
       <x:c r="G3" s="5"/>
@@ -6438,19 +6452,19 @@
     </x:row>
     <x:row r="4" ht="63.95000076293945" customHeight="1">
       <x:c r="A4" s="5" t="s">
-        <x:v>573</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B4" s="11" t="s">
-        <x:v>578</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>579</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>580</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>581</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="F4" s="5"/>
       <x:c r="G4" s="5"/>
@@ -6462,24 +6476,24 @@
     </x:row>
     <x:row r="5" ht="63.95000076293945" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>582</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B5" s="11" t="s">
-        <x:v>583</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="C5" s="5"/>
       <x:c r="D5" s="5" t="s">
-        <x:v>584</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>585</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5" t="s">
-        <x:v>586</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="H5" s="5" t="s">
-        <x:v>587</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="I5" s="5">
         <x:v>1</x:v>
@@ -6488,24 +6502,24 @@
     </x:row>
     <x:row r="6" ht="63.95000076293945" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>582</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B6" s="11" t="s">
-        <x:v>588</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="C6" s="5"/>
       <x:c r="D6" s="5" t="s">
-        <x:v>589</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>590</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5" t="s">
-        <x:v>591</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="H6" s="5" t="s">
-        <x:v>592</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="I6" s="5">
         <x:v>2</x:v>
@@ -6514,24 +6528,24 @@
     </x:row>
     <x:row r="7" ht="63.95000076293945" customHeight="1">
       <x:c r="A7" s="5" t="s">
-        <x:v>582</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B7" s="11" t="s">
-        <x:v>593</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="C7" s="5"/>
       <x:c r="D7" s="5" t="s">
-        <x:v>594</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>595</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="F7" s="5"/>
       <x:c r="G7" s="5" t="s">
-        <x:v>596</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="H7" s="5" t="s">
-        <x:v>597</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="I7" s="5">
         <x:v>3</x:v>
@@ -6540,24 +6554,24 @@
     </x:row>
     <x:row r="8" ht="63.95000076293945" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>582</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B8" s="11" t="s">
-        <x:v>598</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="C8" s="5"/>
       <x:c r="D8" s="5" t="s">
-        <x:v>599</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>600</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="F8" s="5"/>
       <x:c r="G8" s="5" t="s">
-        <x:v>601</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="H8" s="5" t="s">
-        <x:v>602</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="I8" s="5">
         <x:v>4</x:v>
@@ -6566,24 +6580,24 @@
     </x:row>
     <x:row r="9" ht="63.95000076293945" customHeight="1">
       <x:c r="A9" s="5" t="s">
-        <x:v>582</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B9" s="11" t="s">
-        <x:v>603</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="C9" s="5"/>
       <x:c r="D9" s="5" t="s">
-        <x:v>604</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>605</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="F9" s="5"/>
       <x:c r="G9" s="5" t="s">
-        <x:v>606</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="H9" s="5" t="s">
-        <x:v>607</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="I9" s="5">
         <x:v>5</x:v>
@@ -6592,24 +6606,24 @@
     </x:row>
     <x:row r="10" ht="63.95000076293945" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>608</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B10" s="11" t="s">
-        <x:v>609</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="C10" s="5"/>
       <x:c r="D10" s="5" t="s">
-        <x:v>610</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>611</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="F10" s="5"/>
       <x:c r="G10" s="5" t="s">
-        <x:v>612</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="H10" s="5" t="s">
-        <x:v>613</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="I10" s="5">
         <x:v>1</x:v>
@@ -6618,24 +6632,24 @@
     </x:row>
     <x:row r="11" ht="63.95000076293945" customHeight="1">
       <x:c r="A11" s="5" t="s">
-        <x:v>608</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B11" s="11" t="s">
-        <x:v>614</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="C11" s="5"/>
       <x:c r="D11" s="5" t="s">
-        <x:v>615</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>616</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="F11" s="5"/>
       <x:c r="G11" s="5" t="s">
-        <x:v>617</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="H11" s="5" t="s">
-        <x:v>618</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="I11" s="5">
         <x:v>2</x:v>
@@ -6644,24 +6658,24 @@
     </x:row>
     <x:row r="12" ht="63.95000076293945" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>608</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B12" s="11" t="s">
-        <x:v>619</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="C12" s="5"/>
       <x:c r="D12" s="5" t="s">
-        <x:v>620</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>621</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="F12" s="5"/>
       <x:c r="G12" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="H12" s="5" t="s">
-        <x:v>623</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="I12" s="5">
         <x:v>3</x:v>
@@ -6670,24 +6684,24 @@
     </x:row>
     <x:row r="13" ht="63.95000076293945" customHeight="1">
       <x:c r="A13" s="5" t="s">
-        <x:v>608</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B13" s="11" t="s">
-        <x:v>624</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="C13" s="5"/>
       <x:c r="D13" s="5" t="s">
-        <x:v>625</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>626</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="F13" s="5"/>
       <x:c r="G13" s="5" t="s">
-        <x:v>627</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="H13" s="5" t="s">
-        <x:v>628</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="I13" s="5">
         <x:v>4</x:v>
@@ -6696,24 +6710,24 @@
     </x:row>
     <x:row r="14" ht="63.95000076293945" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>608</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B14" s="11" t="s">
-        <x:v>629</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="C14" s="5"/>
       <x:c r="D14" s="5" t="s">
-        <x:v>630</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>631</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="F14" s="5"/>
       <x:c r="G14" s="5" t="s">
-        <x:v>632</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="H14" s="5" t="s">
-        <x:v>633</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="I14" s="5">
         <x:v>5</x:v>
@@ -6722,109 +6736,109 @@
     </x:row>
     <x:row r="15" ht="63.95000076293945" customHeight="1">
       <x:c r="A15" s="5" t="s">
-        <x:v>634</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="B15" s="11" t="s">
-        <x:v>635</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
         <x:v>381</x:v>
       </x:c>
       <x:c r="D15" s="5" t="s">
-        <x:v>636</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>637</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="F15" s="5" t="s">
         <x:v>382</x:v>
       </x:c>
       <x:c r="G15" s="5" t="s">
-        <x:v>638</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="H15" s="5" t="s">
-        <x:v>639</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="I15" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J15" s="7" t="s">
-        <x:v>640</x:v>
+        <x:v>604</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="63.95000076293945" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>634</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="B16" s="11" t="s">
-        <x:v>641</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
         <x:v>396</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>642</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>643</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
         <x:v>382</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
-        <x:v>644</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="H16" s="5" t="s">
-        <x:v>645</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="I16" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="J16" s="7" t="s">
-        <x:v>646</x:v>
+        <x:v>610</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="63.95000076293945" customHeight="1">
       <x:c r="A17" s="5" t="s">
-        <x:v>634</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="B17" s="11" t="s">
-        <x:v>647</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="C17" s="5" t="s">
         <x:v>410</x:v>
       </x:c>
       <x:c r="D17" s="5" t="s">
-        <x:v>648</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>649</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="F17" s="5" t="s">
         <x:v>382</x:v>
       </x:c>
       <x:c r="G17" s="5" t="s">
-        <x:v>650</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="H17" s="5" t="s">
-        <x:v>651</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="I17" s="5">
         <x:v>3</x:v>
       </x:c>
       <x:c r="J17" s="7" t="s">
-        <x:v>652</x:v>
+        <x:v>616</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="63.95000076293945" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>653</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="B18" s="11" t="s">
-        <x:v>654</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>655</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
         <x:v>49</x:v>
@@ -6836,10 +6850,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="G18" s="5" t="s">
-        <x:v>656</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="H18" s="5" t="s">
-        <x:v>656</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="I18" s="5">
         <x:v>1</x:v>
@@ -6848,13 +6862,13 @@
     </x:row>
     <x:row r="19" ht="63.95000076293945" customHeight="1">
       <x:c r="A19" s="5" t="s">
-        <x:v>653</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="B19" s="11" t="s">
-        <x:v>657</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D19" s="5" t="s">
         <x:v>60</x:v>
@@ -6866,10 +6880,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
-        <x:v>659</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="H19" s="5" t="s">
-        <x:v>659</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="I19" s="5">
         <x:v>2</x:v>
@@ -6878,13 +6892,13 @@
     </x:row>
     <x:row r="20" ht="63.95000076293945" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>653</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="B20" s="11" t="s">
-        <x:v>660</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D20" s="5" t="s">
         <x:v>68</x:v>
@@ -6896,10 +6910,10 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
-        <x:v>661</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="H20" s="5" t="s">
-        <x:v>661</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="I20" s="5">
         <x:v>3</x:v>
@@ -6908,13 +6922,13 @@
     </x:row>
     <x:row r="21" ht="63.95000076293945" customHeight="1">
       <x:c r="A21" s="5" t="s">
-        <x:v>653</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="B21" s="11" t="s">
-        <x:v>662</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="C21" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D21" s="5" t="s">
         <x:v>93</x:v>
@@ -6926,10 +6940,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="G21" s="5" t="s">
-        <x:v>663</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="H21" s="5" t="s">
-        <x:v>663</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="I21" s="5">
         <x:v>4</x:v>
@@ -6938,13 +6952,13 @@
     </x:row>
     <x:row r="22" ht="63.95000076293945" customHeight="1">
       <x:c r="A22" s="5" t="s">
-        <x:v>653</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="B22" s="11" t="s">
-        <x:v>664</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>665</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
         <x:v>110</x:v>
@@ -6956,10 +6970,10 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="G22" s="5" t="s">
-        <x:v>666</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="H22" s="5" t="s">
-        <x:v>666</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="I22" s="5">
         <x:v>5</x:v>
@@ -6968,13 +6982,13 @@
     </x:row>
     <x:row r="23" ht="63.95000076293945" customHeight="1">
       <x:c r="A23" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="B23" s="11" t="s">
-        <x:v>668</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>655</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="D23" s="5" t="s">
         <x:v>238</x:v>
@@ -6983,13 +6997,13 @@
         <x:v>238</x:v>
       </x:c>
       <x:c r="F23" s="5" t="s">
-        <x:v>669</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="G23" s="5" t="s">
-        <x:v>670</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="H23" s="5" t="s">
-        <x:v>670</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="I23" s="5">
         <x:v>1</x:v>
@@ -6998,13 +7012,13 @@
     </x:row>
     <x:row r="24" ht="63.95000076293945" customHeight="1">
       <x:c r="A24" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="B24" s="11" t="s">
-        <x:v>671</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D24" s="5" t="s">
         <x:v>244</x:v>
@@ -7013,13 +7027,13 @@
         <x:v>244</x:v>
       </x:c>
       <x:c r="F24" s="5" t="s">
-        <x:v>672</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="G24" s="5" t="s">
-        <x:v>673</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="H24" s="5" t="s">
-        <x:v>673</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="I24" s="5">
         <x:v>2</x:v>
@@ -7028,13 +7042,13 @@
     </x:row>
     <x:row r="25" ht="63.95000076293945" customHeight="1">
       <x:c r="A25" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="B25" s="11" t="s">
-        <x:v>674</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
         <x:v>272</x:v>
@@ -7043,13 +7057,13 @@
         <x:v>272</x:v>
       </x:c>
       <x:c r="F25" s="5" t="s">
-        <x:v>675</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="G25" s="5" t="s">
-        <x:v>676</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="H25" s="5" t="s">
-        <x:v>676</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="I25" s="5">
         <x:v>3</x:v>
@@ -7058,13 +7072,13 @@
     </x:row>
     <x:row r="26" ht="63.95000076293945" customHeight="1">
       <x:c r="A26" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="B26" s="11" t="s">
-        <x:v>677</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D26" s="5" t="s">
         <x:v>282</x:v>
@@ -7073,13 +7087,13 @@
         <x:v>282</x:v>
       </x:c>
       <x:c r="F26" s="5" t="s">
-        <x:v>678</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="G26" s="5" t="s">
-        <x:v>679</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="H26" s="5" t="s">
-        <x:v>679</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="I26" s="5">
         <x:v>4</x:v>
@@ -7088,13 +7102,13 @@
     </x:row>
     <x:row r="27" ht="63.95000076293945" customHeight="1">
       <x:c r="A27" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="B27" s="11" t="s">
-        <x:v>680</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="C27" s="5" t="s">
-        <x:v>665</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="D27" s="5" t="s">
         <x:v>255</x:v>
@@ -7103,13 +7117,13 @@
         <x:v>255</x:v>
       </x:c>
       <x:c r="F27" s="5" t="s">
-        <x:v>681</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="G27" s="5" t="s">
-        <x:v>682</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="H27" s="5" t="s">
-        <x:v>682</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="I27" s="5">
         <x:v>5</x:v>
@@ -7118,24 +7132,24 @@
     </x:row>
     <x:row r="28" ht="63.95000076293945" customHeight="1">
       <x:c r="A28" s="5" t="s">
-        <x:v>683</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="B28" s="11" t="s">
-        <x:v>684</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="C28" s="5"/>
       <x:c r="D28" s="5" t="s">
-        <x:v>685</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="E28" s="5" t="s">
-        <x:v>686</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="F28" s="5"/>
       <x:c r="G28" s="5" t="s">
-        <x:v>687</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="H28" s="5" t="s">
-        <x:v>688</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="I28" s="5">
         <x:v>1</x:v>
@@ -7144,10 +7158,10 @@
     </x:row>
     <x:row r="29" ht="63.95000076293945" customHeight="1">
       <x:c r="A29" s="5" t="s">
-        <x:v>683</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="B29" s="11" t="s">
-        <x:v>689</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="C29" s="5"/>
       <x:c r="D29" s="5" t="s">
@@ -7158,10 +7172,10 @@
       </x:c>
       <x:c r="F29" s="5"/>
       <x:c r="G29" s="5" t="s">
-        <x:v>690</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="H29" s="5" t="s">
-        <x:v>691</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="I29" s="5">
         <x:v>2</x:v>
@@ -7170,10 +7184,10 @@
     </x:row>
     <x:row r="30" ht="63.95000076293945" customHeight="1">
       <x:c r="A30" s="5" t="s">
-        <x:v>683</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="B30" s="11" t="s">
-        <x:v>692</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="C30" s="5"/>
       <x:c r="D30" s="5" t="s">
@@ -7184,10 +7198,10 @@
       </x:c>
       <x:c r="F30" s="5"/>
       <x:c r="G30" s="5" t="s">
-        <x:v>693</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="H30" s="5" t="s">
-        <x:v>694</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="I30" s="5">
         <x:v>3</x:v>
@@ -7196,10 +7210,10 @@
     </x:row>
     <x:row r="31" ht="63.95000076293945" customHeight="1">
       <x:c r="A31" s="5" t="s">
-        <x:v>683</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="B31" s="11" t="s">
-        <x:v>695</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="C31" s="5"/>
       <x:c r="D31" s="5" t="s">
@@ -7210,10 +7224,10 @@
       </x:c>
       <x:c r="F31" s="5"/>
       <x:c r="G31" s="5" t="s">
-        <x:v>696</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="H31" s="5" t="s">
-        <x:v>697</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="I31" s="5">
         <x:v>4</x:v>
@@ -7222,10 +7236,10 @@
     </x:row>
     <x:row r="32" ht="63.95000076293945" customHeight="1">
       <x:c r="A32" s="5" t="s">
-        <x:v>683</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="B32" s="11" t="s">
-        <x:v>698</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="C32" s="5"/>
       <x:c r="D32" s="5" t="s">
@@ -7236,10 +7250,10 @@
       </x:c>
       <x:c r="F32" s="5"/>
       <x:c r="G32" s="5" t="s">
-        <x:v>699</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="H32" s="5" t="s">
-        <x:v>700</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="I32" s="5">
         <x:v>5</x:v>
@@ -7248,13 +7262,13 @@
     </x:row>
     <x:row r="33" ht="63.95000076293945" customHeight="1">
       <x:c r="A33" s="5" t="s">
-        <x:v>701</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="B33" s="11" t="s">
-        <x:v>702</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="C33" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D33" s="5" t="s">
         <x:v>296</x:v>
@@ -7264,10 +7278,10 @@
       </x:c>
       <x:c r="F33" s="5"/>
       <x:c r="G33" s="5" t="s">
-        <x:v>703</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
-        <x:v>703</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="I33" s="5">
         <x:v>1</x:v>
@@ -7276,13 +7290,13 @@
     </x:row>
     <x:row r="34" ht="63.95000076293945" customHeight="1">
       <x:c r="A34" s="5" t="s">
-        <x:v>701</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="B34" s="11" t="s">
-        <x:v>704</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="C34" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="D34" s="5" t="s">
         <x:v>316</x:v>
@@ -7292,10 +7306,10 @@
       </x:c>
       <x:c r="F34" s="5"/>
       <x:c r="G34" s="5" t="s">
-        <x:v>705</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="H34" s="5" t="s">
-        <x:v>705</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="I34" s="5">
         <x:v>2</x:v>
@@ -7304,13 +7318,13 @@
     </x:row>
     <x:row r="35" ht="63.95000076293945" customHeight="1">
       <x:c r="A35" s="5" t="s">
-        <x:v>701</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="B35" s="11" t="s">
-        <x:v>706</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>707</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="D35" s="5" t="s">
         <x:v>302</x:v>
@@ -7320,10 +7334,10 @@
       </x:c>
       <x:c r="F35" s="5"/>
       <x:c r="G35" s="5" t="s">
-        <x:v>708</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
-        <x:v>708</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="I35" s="5">
         <x:v>3</x:v>
@@ -7332,13 +7346,13 @@
     </x:row>
     <x:row r="36" ht="63.95000076293945" customHeight="1">
       <x:c r="A36" s="5" t="s">
-        <x:v>701</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="B36" s="11" t="s">
-        <x:v>709</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="C36" s="5" t="s">
-        <x:v>710</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="D36" s="5" t="s">
         <x:v>309</x:v>
@@ -7348,10 +7362,10 @@
       </x:c>
       <x:c r="F36" s="5"/>
       <x:c r="G36" s="5" t="s">
-        <x:v>711</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="H36" s="5" t="s">
-        <x:v>711</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="I36" s="5">
         <x:v>4</x:v>
@@ -7361,7 +7375,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83e1f7eb20bd42a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30ff6c7d2c3846a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7383,13 +7397,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>712</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>713</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>714</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
         <x:v>45</x:v>
@@ -7406,13 +7420,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B2" s="4" t="s">
-        <x:v>715</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="C2" s="4" t="s">
-        <x:v>716</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="D2" s="4" t="s">
-        <x:v>717</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
         <x:v>16</x:v>
@@ -7421,7 +7435,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="G2" s="6" t="s">
-        <x:v>718</x:v>
+        <x:v>682</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -7429,16 +7443,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>719</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>720</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="D3" s="5" t="s">
         <x:v>20</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>569</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="F3" s="5" t="s">
         <x:v>57</x:v>
@@ -7447,19 +7461,19 @@
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="11" t="s">
-        <x:v>721</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>722</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>722</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>723</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>569</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="F4" s="5" t="s">
         <x:v>57</x:v>
@@ -7468,19 +7482,19 @@
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>724</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>725</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>725</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>726</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>569</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="F5" s="5" t="s">
         <x:v>57</x:v>
@@ -7489,16 +7503,16 @@
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>727</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
         <x:v>382</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>728</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>729</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
         <x:v>366</x:v>
@@ -7510,133 +7524,133 @@
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>730</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>731</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>731</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="D7" s="5"/>
       <x:c r="E7" s="5" t="s">
-        <x:v>569</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="F7" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
       <x:c r="G7" s="7" t="s">
-        <x:v>732</x:v>
+        <x:v>696</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>733</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>734</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>734</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="D8" s="5"/>
       <x:c r="E8" s="5" t="s">
-        <x:v>569</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="F8" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
       <x:c r="G8" s="7" t="s">
-        <x:v>732</x:v>
+        <x:v>696</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>735</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>736</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="C9" s="5"/>
       <x:c r="D9" s="5" t="s">
-        <x:v>737</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>738</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="F9" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>739</x:v>
+        <x:v>703</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>740</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>741</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="C10" s="5"/>
       <x:c r="D10" s="5" t="s">
-        <x:v>742</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>738</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="F10" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>739</x:v>
+        <x:v>703</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>743</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="B11" s="5"/>
       <x:c r="C11" s="5" t="s">
-        <x:v>744</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>745</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>738</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="F11" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>746</x:v>
+        <x:v>710</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>747</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="B12" s="5"/>
       <x:c r="C12" s="5" t="s">
-        <x:v>748</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>749</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>738</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="F12" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G12" s="7" t="s">
-        <x:v>746</x:v>
+        <x:v>710</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="11" t="s">
-        <x:v>750</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
         <x:v>49</x:v>
@@ -7648,7 +7662,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F13" s="5" t="s">
         <x:v>57</x:v>
@@ -7657,7 +7671,7 @@
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="11" t="s">
-        <x:v>752</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
         <x:v>60</x:v>
@@ -7669,7 +7683,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
         <x:v>57</x:v>
@@ -7678,7 +7692,7 @@
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="11" t="s">
-        <x:v>753</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
         <x:v>68</x:v>
@@ -7690,7 +7704,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F15" s="5" t="s">
         <x:v>57</x:v>
@@ -7699,7 +7713,7 @@
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>754</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
         <x:v>77</x:v>
@@ -7711,7 +7725,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
         <x:v>57</x:v>
@@ -7720,7 +7734,7 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="11" t="s">
-        <x:v>755</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
         <x:v>86</x:v>
@@ -7732,7 +7746,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F17" s="5" t="s">
         <x:v>57</x:v>
@@ -7741,7 +7755,7 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>756</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
         <x:v>93</x:v>
@@ -7753,7 +7767,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F18" s="5" t="s">
         <x:v>57</x:v>
@@ -7762,7 +7776,7 @@
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="11" t="s">
-        <x:v>757</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
         <x:v>103</x:v>
@@ -7774,7 +7788,7 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="E19" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F19" s="5" t="s">
         <x:v>57</x:v>
@@ -7783,7 +7797,7 @@
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="11" t="s">
-        <x:v>758</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
         <x:v>110</x:v>
@@ -7795,7 +7809,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F20" s="5" t="s">
         <x:v>57</x:v>
@@ -7804,7 +7818,7 @@
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="11" t="s">
-        <x:v>759</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
         <x:v>119</x:v>
@@ -7816,7 +7830,7 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="E21" s="5" t="s">
-        <x:v>751</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F21" s="5" t="s">
         <x:v>57</x:v>
@@ -7825,7 +7839,7 @@
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="11" t="s">
-        <x:v>760</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
         <x:v>238</x:v>
@@ -7846,7 +7860,7 @@
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="11" t="s">
-        <x:v>761</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
         <x:v>244</x:v>
@@ -7867,7 +7881,7 @@
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="11" t="s">
-        <x:v>762</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
         <x:v>255</x:v>
@@ -7888,7 +7902,7 @@
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="11" t="s">
-        <x:v>763</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
         <x:v>272</x:v>
@@ -7909,7 +7923,7 @@
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="11" t="s">
-        <x:v>764</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
         <x:v>278</x:v>
@@ -7939,7 +7953,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R071f350b693d4188"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3747c106ebca47b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
content: add SATURN live gallery photo
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rc1a106a8df0c4cb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R391d607e158d4fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R7dc5758150e84b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R48d448f6a1874802"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="Ra27ce088b7d34d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R088e75820ca74747"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="Re4943b696a474e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="Rfca71930f7bf4b2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R25b9f0d4ce644078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="R91f8832b79a24e19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="Ra0927586327d45ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="Rb3b559e7e8d44196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R462a179668214e09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R276d338a2791405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R6446dde2cfb34a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R4b0e57caa75f4491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R9dd47217fd20473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R1daa293334674a4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2595,8 +2595,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J42" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:J42"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J43" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J43"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="date"/>
@@ -2989,7 +2989,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2df0ca8d5a25459e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R045544da664d459a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3602,7 +3602,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4d48cb48bc14033"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a70942ef7d4926"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4257,7 +4257,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2092621003fb4748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd64ac54cfb3f4f08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4663,7 +4663,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f8dcf4ea3aa40ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50d82dcff0df4e6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5067,7 +5067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a73f7bec4fe44a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553dc3e3fe004436"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5306,7 +5306,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e0c81c7a9a0428c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eeaf91720974861"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6341,6 +6341,30 @@
       </x:c>
       <x:c r="J42"/>
     </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>gallery_042</x:v>
+      </x:c>
+      <x:c r="B43" s="17" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>SATURN live</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>SATURN 演出</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>assets/albums-optimized/20260912_SATURN%20%E6%BC%94%E5%87%BA.webp</x:v>
+      </x:c>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
+      <x:c r="I43" t="str">
+        <x:v>20260912_SATURN 演出.jpg</x:v>
+      </x:c>
+      <x:c r="J43"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F2:F37">
@@ -6349,7 +6373,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61b6a7d90cdc4a7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f58cfe67e604e87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7375,7 +7399,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30ff6c7d2c3846a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2bf5b5d9fca49b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7953,7 +7977,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3747c106ebca47b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e3101ca1cd340b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
content: update academic honors and gallery
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="R91f8832b79a24e19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="Ra0927586327d45ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="Rb3b559e7e8d44196"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R462a179668214e09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R276d338a2791405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R6446dde2cfb34a61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R4b0e57caa75f4491"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R9dd47217fd20473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R1daa293334674a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Radbd3e8e219948e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="Rdd80c23f3ec34e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="Rbd2b160797b54d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R275538baa40549e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R0e9b6e0a1982471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="Rff96d16248634970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R896606a52cd744c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R9a696770eb1f41b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="Rd0a326455d314de1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1068,12 +1068,6 @@
     <x:t xml:space="preserve">Conference paper award</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Awarded for an outstanding conference paper presented at KMEMS 2025.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">因在 KMEMS 2025 发表的优秀会议论文获奖。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">award_006</x:t>
   </x:si>
   <x:si>
@@ -1081,12 +1075,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">KSS 2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Awarded for an best conference paper presented at KSS 2025.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">因在 KSS 2025 发表的优秀会议论文获奖。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">award_007</x:t>
@@ -2550,8 +2538,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="awardsTable" displayName="awardsTable" ref="A1:J13">
-  <x:autoFilter ref="A1:J13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="awardsTable" displayName="awardsTable" ref="A1:J14" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J14"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="year"/>
@@ -2595,8 +2583,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J43" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:J43"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J44" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J44"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="date"/>
@@ -2989,7 +2977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R045544da664d459a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77aba52755e94f36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3602,7 +3590,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a70942ef7d4926"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc47d3b7dddc84c08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4257,7 +4245,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd64ac54cfb3f4f08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0cef20cf2b462f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4663,7 +4651,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50d82dcff0df4e6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8eb1f759cb194c04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4853,26 +4841,26 @@
       <x:c r="G6" s="5" t="s">
         <x:v>252</x:v>
       </x:c>
-      <x:c r="H6" s="5" t="s">
-        <x:v>325</x:v>
-      </x:c>
-      <x:c r="I6" s="5" t="s">
-        <x:v>326</x:v>
+      <x:c r="H6" s="5" t="str">
+        <x:v>Awarded for an outstanding conference paper presented at KMEMS 2025 (The Society of Micro and Nano Systems).</x:v>
+      </x:c>
+      <x:c r="I6" s="5" t="str">
+        <x:v>因在 KMEMS 2025 (The Society of Micro and Nano Systems) 上发表的优秀会议论文而获奖。</x:v>
       </x:c>
       <x:c r="J6" s="7"/>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B7" s="5">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>328</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>328</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
         <x:v>317</x:v>
@@ -4881,183 +4869,213 @@
         <x:v>324</x:v>
       </x:c>
       <x:c r="G7" s="5" t="s">
-        <x:v>329</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="s">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="I7" s="14" t="s">
-        <x:v>331</x:v>
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="H7" s="5" t="str">
+        <x:v>Awarded for an best conference paper presented at KSS 2025 (Conference of the Korean Sensors Society).</x:v>
+      </x:c>
+      <x:c r="I7" s="14" t="str">
+        <x:v>因在 KSS 2025 (Conference of the Korean Sensors Society) 上发表的最佳会议论文而获奖。</x:v>
       </x:c>
       <x:c r="J7" s="7"/>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>332</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="B8" s="5">
         <x:v>2021</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>333</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="D8" s="5" t="s">
-        <x:v>334</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F8" s="5" t="s">
-        <x:v>336</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5" t="s">
-        <x:v>337</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="I8" s="5" t="s">
-        <x:v>338</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="J8" s="7"/>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>339</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="B9" s="5">
         <x:v>2020</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>340</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="D9" s="5" t="s">
-        <x:v>341</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F9" s="5" t="s">
-        <x:v>342</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="5" t="s">
-        <x:v>343</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="I9" s="5" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="J9" s="7"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="B10" s="5">
         <x:v>2020</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>346</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>347</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F10" s="5" t="s">
-        <x:v>348</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="G10" s="5"/>
       <x:c r="H10" s="5" t="s">
-        <x:v>348</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="I10" s="5" t="s">
-        <x:v>349</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="J10" s="7"/>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>350</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="B11" s="5">
         <x:v>2020</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>351</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>352</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F11" s="5" t="s">
-        <x:v>353</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="G11" s="5"/>
       <x:c r="H11" s="5" t="s">
-        <x:v>354</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="I11" s="5" t="s">
-        <x:v>355</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="J11" s="7"/>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>356</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="B12" s="5">
         <x:v>2019</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>357</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>358</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F12" s="5" t="s">
-        <x:v>353</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="G12" s="5"/>
       <x:c r="H12" s="5" t="s">
-        <x:v>359</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="I12" s="5" t="s">
-        <x:v>360</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="J12" s="7"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="11" t="s">
-        <x:v>361</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="B13" s="5">
         <x:v>2019</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>362</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="D13" s="5" t="s">
-        <x:v>363</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>335</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F13" s="5" t="s">
-        <x:v>336</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="G13" s="5"/>
       <x:c r="H13" s="5" t="s">
-        <x:v>337</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="I13" s="5" t="s">
-        <x:v>364</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="J13" s="7"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>award_013</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Best Poster Presentation Award, JCK MEMS/NEMS 2026</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Best Poster Presentation Award, JCK MEMS/NEMS 2026</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>academic_honor</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Conference presentation award</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>JCK MEMS/NEMS 2026</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Awarded for an best conference paper presented at JCK MEMS/NEMS 2026 (Japan–China–Korea Joint Conference on MEMS/NEMS).</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Awarded for an best conference paper presented at JCK MEMS/NEMS 2026 (Japan–China–Korea Joint Conference on MEMS/NEMS).</x:v>
+      </x:c>
+      <x:c r="J14"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -5067,7 +5085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553dc3e3fe004436"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1f1eb5179214f77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5097,43 +5115,43 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="s">
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="F1" s="2" t="s">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="G1" s="2" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="H1" s="2" t="s">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="E1" s="2" t="s">
+      <x:c r="I1" s="2" t="s">
         <x:v>366</x:v>
       </x:c>
-      <x:c r="F1" s="2" t="s">
+      <x:c r="J1" s="2" t="s">
         <x:v>367</x:v>
       </x:c>
-      <x:c r="G1" s="2" t="s">
+      <x:c r="K1" s="2" t="s">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="H1" s="2" t="s">
+      <x:c r="L1" s="2" t="s">
         <x:v>369</x:v>
       </x:c>
-      <x:c r="I1" s="2" t="s">
+      <x:c r="M1" s="2" t="s">
         <x:v>370</x:v>
       </x:c>
-      <x:c r="J1" s="2" t="s">
+      <x:c r="N1" s="2" t="s">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="K1" s="2" t="s">
+      <x:c r="O1" s="2" t="s">
         <x:v>372</x:v>
       </x:c>
-      <x:c r="L1" s="2" t="s">
+      <x:c r="P1" s="2" t="s">
         <x:v>373</x:v>
-      </x:c>
-      <x:c r="M1" s="2" t="s">
-        <x:v>374</x:v>
-      </x:c>
-      <x:c r="N1" s="2" t="s">
-        <x:v>375</x:v>
-      </x:c>
-      <x:c r="O1" s="2" t="s">
-        <x:v>376</x:v>
-      </x:c>
-      <x:c r="P1" s="2" t="s">
-        <x:v>377</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="s">
         <x:v>3</x:v>
@@ -5141,46 +5159,46 @@
     </x:row>
     <x:row r="2" ht="63.95000076293945" customHeight="1">
       <x:c r="A2" s="10" t="s">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="B2" s="4" t="s">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="C2" s="4" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="s">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="E2" s="4" t="s">
         <x:v>378</x:v>
       </x:c>
-      <x:c r="B2" s="4" t="s">
+      <x:c r="F2" s="4" t="s">
         <x:v>379</x:v>
       </x:c>
-      <x:c r="C2" s="4" t="s">
+      <x:c r="G2" s="4" t="s">
         <x:v>380</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="s">
+      <x:c r="H2" s="4" t="s">
         <x:v>381</x:v>
       </x:c>
-      <x:c r="E2" s="4" t="s">
+      <x:c r="I2" s="4" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="F2" s="4" t="s">
+      <x:c r="J2" s="4" t="s">
         <x:v>383</x:v>
       </x:c>
-      <x:c r="G2" s="4" t="s">
+      <x:c r="K2" s="4" t="s">
         <x:v>384</x:v>
       </x:c>
-      <x:c r="H2" s="4" t="s">
+      <x:c r="L2" s="4" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="I2" s="4" t="s">
+      <x:c r="M2" s="4" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="J2" s="4" t="s">
+      <x:c r="N2" s="4" t="s">
         <x:v>387</x:v>
-      </x:c>
-      <x:c r="K2" s="4" t="s">
-        <x:v>388</x:v>
-      </x:c>
-      <x:c r="L2" s="4" t="s">
-        <x:v>389</x:v>
-      </x:c>
-      <x:c r="M2" s="4" t="s">
-        <x:v>390</x:v>
-      </x:c>
-      <x:c r="N2" s="4" t="s">
-        <x:v>391</x:v>
       </x:c>
       <x:c r="O2" s="4" t="s">
         <x:v>57</x:v>
@@ -5189,51 +5207,51 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="s">
-        <x:v>392</x:v>
+        <x:v>388</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="63.95000076293945" customHeight="1">
       <x:c r="A3" s="11" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="s">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="E3" s="5" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="F3" s="5" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="s">
+      <x:c r="G3" s="5" t="s">
         <x:v>394</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="s">
+      <x:c r="H3" s="5" t="s">
         <x:v>395</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="s">
+      <x:c r="I3" s="5" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="F3" s="5" t="s">
+      <x:c r="J3" s="5" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="G3" s="5" t="s">
+      <x:c r="K3" s="5" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="H3" s="5" t="s">
+      <x:c r="L3" s="5" t="s">
         <x:v>399</x:v>
       </x:c>
-      <x:c r="I3" s="5" t="s">
+      <x:c r="M3" s="5" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="J3" s="5" t="s">
+      <x:c r="N3" s="5" t="s">
         <x:v>401</x:v>
-      </x:c>
-      <x:c r="K3" s="5" t="s">
-        <x:v>402</x:v>
-      </x:c>
-      <x:c r="L3" s="5" t="s">
-        <x:v>403</x:v>
-      </x:c>
-      <x:c r="M3" s="5" t="s">
-        <x:v>404</x:v>
-      </x:c>
-      <x:c r="N3" s="5" t="s">
-        <x:v>405</x:v>
       </x:c>
       <x:c r="O3" s="5" t="s">
         <x:v>57</x:v>
@@ -5242,51 +5260,51 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q3" s="7" t="s">
-        <x:v>406</x:v>
+        <x:v>402</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="63.95000076293945" customHeight="1">
       <x:c r="A4" s="11" t="s">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="F4" s="5" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="s">
+      <x:c r="G4" s="5" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
+      <x:c r="H4" s="5" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="s">
+      <x:c r="I4" s="5" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="F4" s="5" t="s">
+      <x:c r="J4" s="5" t="s">
         <x:v>411</x:v>
       </x:c>
-      <x:c r="G4" s="5" t="s">
+      <x:c r="K4" s="5" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="H4" s="5" t="s">
+      <x:c r="L4" s="5" t="s">
         <x:v>413</x:v>
       </x:c>
-      <x:c r="I4" s="5" t="s">
+      <x:c r="M4" s="5" t="s">
         <x:v>414</x:v>
       </x:c>
-      <x:c r="J4" s="5" t="s">
+      <x:c r="N4" s="5" t="s">
         <x:v>415</x:v>
-      </x:c>
-      <x:c r="K4" s="5" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="L4" s="5" t="s">
-        <x:v>417</x:v>
-      </x:c>
-      <x:c r="M4" s="5" t="s">
-        <x:v>418</x:v>
-      </x:c>
-      <x:c r="N4" s="5" t="s">
-        <x:v>419</x:v>
       </x:c>
       <x:c r="O4" s="5" t="s">
         <x:v>57</x:v>
@@ -5295,7 +5313,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q4" s="7" t="s">
-        <x:v>420</x:v>
+        <x:v>416</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5306,7 +5324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eeaf91720974861"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e9903a50edc455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5339,7 +5357,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>375</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
         <x:v>290</x:v>
@@ -5351,7 +5369,7 @@
         <x:v>294</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>421</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="J1" s="3" t="s">
         <x:v>3</x:v>
@@ -5359,7 +5377,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="10" t="s">
-        <x:v>422</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="B2" s="12">
         <x:v>46157</x:v>
@@ -5371,19 +5389,19 @@
         <x:v>济州松岳山日出</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
-        <x:v>423</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4" t="s">
-        <x:v>424</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="J2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="11" t="s">
-        <x:v>425</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="B3" s="13">
         <x:v>46110</x:v>
@@ -5395,19 +5413,19 @@
         <x:v>大变蛋糕人</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>426</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="F3" s="5"/>
       <x:c r="G3" s="5"/>
       <x:c r="H3" s="5"/>
       <x:c r="I3" s="5" t="s">
-        <x:v>427</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="J3" s="7"/>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="11" t="s">
-        <x:v>428</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="B4" s="13">
         <x:v>46109</x:v>
@@ -5419,19 +5437,19 @@
         <x:v>济州卡丁车</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>429</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="F4" s="5"/>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5" t="s">
-        <x:v>430</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="J4" s="7"/>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>431</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="B5" s="13">
         <x:v>46076</x:v>
@@ -5443,19 +5461,19 @@
         <x:v>马头人滑雪</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>432</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5" t="s">
-        <x:v>433</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="J5" s="7"/>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>434</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="B6" s="13">
         <x:v>46054</x:v>
@@ -5467,19 +5485,19 @@
         <x:v>智异山顶</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>435</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5" t="s">
-        <x:v>436</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="J6" s="7"/>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="B7" s="13">
         <x:v>46028</x:v>
@@ -5491,19 +5509,19 @@
         <x:v>BK+统营</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="F7" s="5"/>
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5" t="s">
-        <x:v>439</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="J7" s="7"/>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="B8" s="13">
         <x:v>45987</x:v>
@@ -5515,19 +5533,19 @@
         <x:v>大变圣诞老人</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>441</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="F8" s="5"/>
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5" t="s">
-        <x:v>442</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="J8" s="7"/>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>443</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="B9" s="13">
         <x:v>45976</x:v>
@@ -5539,19 +5557,19 @@
         <x:v>釜山烟花节</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>444</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="F9" s="5"/>
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5" t="s">
-        <x:v>445</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="J9" s="7"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>446</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="B10" s="13">
         <x:v>45957</x:v>
@@ -5563,19 +5581,19 @@
         <x:v>温哥华SENSORS</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>447</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="F10" s="5"/>
       <x:c r="G10" s="5"/>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5" t="s">
-        <x:v>448</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J10" s="7"/>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>449</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="B11" s="13">
         <x:v>45937</x:v>
@@ -5587,19 +5605,19 @@
         <x:v>米菲70周年</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>450</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="F11" s="5"/>
       <x:c r="G11" s="5"/>
       <x:c r="H11" s="5"/>
       <x:c r="I11" s="5" t="s">
-        <x:v>451</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="J11" s="7"/>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>452</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="B12" s="13">
         <x:v>45932</x:v>
@@ -5611,19 +5629,19 @@
         <x:v>丽水楠哥婚礼</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>453</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="F12" s="5"/>
       <x:c r="G12" s="5"/>
       <x:c r="H12" s="5"/>
       <x:c r="I12" s="5" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="J12" s="7"/>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="11" t="s">
-        <x:v>455</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="B13" s="13">
         <x:v>45897</x:v>
@@ -5635,19 +5653,19 @@
         <x:v>MNTL谭阳</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>456</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="F13" s="5"/>
       <x:c r="G13" s="5"/>
       <x:c r="H13" s="5"/>
       <x:c r="I13" s="5" t="s">
-        <x:v>457</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="J13" s="7"/>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="11" t="s">
-        <x:v>458</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B14" s="13">
         <x:v>45895</x:v>
@@ -5659,19 +5677,19 @@
         <x:v>BK FellowShip 奖学金</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="F14" s="5"/>
       <x:c r="G14" s="5"/>
       <x:c r="H14" s="5"/>
       <x:c r="I14" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="J14" s="7"/>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="11" t="s">
-        <x:v>461</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B15" s="13">
         <x:v>45801</x:v>
@@ -5683,19 +5701,19 @@
         <x:v>Dr.Nomin 聚餐</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>462</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="F15" s="5"/>
       <x:c r="G15" s="5"/>
       <x:c r="H15" s="5"/>
       <x:c r="I15" s="5" t="s">
-        <x:v>463</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="J15" s="7"/>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>464</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B16" s="13">
         <x:v>45781</x:v>
@@ -5707,19 +5725,19 @@
         <x:v>浦项SpaceWalk</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="5"/>
       <x:c r="I16" s="5" t="s">
-        <x:v>466</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="J16" s="7"/>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="11" t="s">
-        <x:v>467</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="B17" s="13">
         <x:v>45744</x:v>
@@ -5731,19 +5749,19 @@
         <x:v>济州枪击</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="F17" s="5"/>
       <x:c r="G17" s="5"/>
       <x:c r="H17" s="5"/>
       <x:c r="I17" s="5" t="s">
-        <x:v>469</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="J17" s="7"/>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>470</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B18" s="13">
         <x:v>45725</x:v>
@@ -5755,19 +5773,19 @@
         <x:v>羽毛球比赛</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>471</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="F18" s="5"/>
       <x:c r="G18" s="5"/>
       <x:c r="H18" s="5"/>
       <x:c r="I18" s="5" t="s">
-        <x:v>472</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="J18" s="7"/>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="11" t="s">
-        <x:v>473</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="B19" s="13">
         <x:v>45715</x:v>
@@ -5779,19 +5797,19 @@
         <x:v>RLRC最佳研究生</x:v>
       </x:c>
       <x:c r="E19" s="5" t="s">
-        <x:v>474</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
       <x:c r="H19" s="5"/>
       <x:c r="I19" s="5" t="s">
-        <x:v>475</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="J19" s="7"/>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="11" t="s">
-        <x:v>476</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="B20" s="13">
         <x:v>45692</x:v>
@@ -5803,19 +5821,19 @@
         <x:v>福州添福</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>477</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="F20" s="5"/>
       <x:c r="G20" s="5"/>
       <x:c r="H20" s="5"/>
       <x:c r="I20" s="5" t="s">
-        <x:v>478</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="J20" s="7"/>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="11" t="s">
-        <x:v>479</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B21" s="13">
         <x:v>45690</x:v>
@@ -5827,19 +5845,19 @@
         <x:v>大变财神</x:v>
       </x:c>
       <x:c r="E21" s="5" t="s">
-        <x:v>480</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="F21" s="5"/>
       <x:c r="G21" s="5"/>
       <x:c r="H21" s="5"/>
       <x:c r="I21" s="5" t="s">
-        <x:v>481</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="J21" s="7"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="11" t="s">
-        <x:v>482</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B22" s="13">
         <x:v>45686</x:v>
@@ -5851,19 +5869,19 @@
         <x:v>杭州径山</x:v>
       </x:c>
       <x:c r="E22" s="5" t="s">
-        <x:v>483</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="F22" s="5"/>
       <x:c r="G22" s="5"/>
       <x:c r="H22" s="5"/>
       <x:c r="I22" s="5" t="s">
-        <x:v>484</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="J22" s="7"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="11" t="s">
-        <x:v>485</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B23" s="13">
         <x:v>45651</x:v>
@@ -5875,19 +5893,19 @@
         <x:v>圣诞节+汉拿山</x:v>
       </x:c>
       <x:c r="E23" s="5" t="s">
-        <x:v>486</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="F23" s="5"/>
       <x:c r="G23" s="5"/>
       <x:c r="H23" s="5"/>
       <x:c r="I23" s="5" t="s">
-        <x:v>487</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="J23" s="7"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="11" t="s">
-        <x:v>488</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="B24" s="13">
         <x:v>45618</x:v>
@@ -5899,19 +5917,19 @@
         <x:v>釜山海上烟花</x:v>
       </x:c>
       <x:c r="E24" s="5" t="s">
-        <x:v>489</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="F24" s="5"/>
       <x:c r="G24" s="5"/>
       <x:c r="H24" s="5"/>
       <x:c r="I24" s="5" t="s">
-        <x:v>490</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="J24" s="7"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="11" t="s">
-        <x:v>491</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="B25" s="13">
         <x:v>45612</x:v>
@@ -5923,19 +5941,19 @@
         <x:v>无等山顶</x:v>
       </x:c>
       <x:c r="E25" s="5" t="s">
-        <x:v>492</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="F25" s="5"/>
       <x:c r="G25" s="5"/>
       <x:c r="H25" s="5"/>
       <x:c r="I25" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="J25" s="7"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="11" t="s">
-        <x:v>494</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B26" s="13">
         <x:v>45507</x:v>
@@ -5947,19 +5965,19 @@
         <x:v>釜山海云台</x:v>
       </x:c>
       <x:c r="E26" s="5" t="s">
-        <x:v>495</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="F26" s="5"/>
       <x:c r="G26" s="5"/>
       <x:c r="H26" s="5"/>
       <x:c r="I26" s="5" t="s">
-        <x:v>496</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="J26" s="7"/>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="11" t="s">
-        <x:v>497</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B27" s="13">
         <x:v>45392</x:v>
@@ -5971,19 +5989,19 @@
         <x:v>动物园</x:v>
       </x:c>
       <x:c r="E27" s="5" t="s">
-        <x:v>498</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F27" s="5"/>
       <x:c r="G27" s="5"/>
       <x:c r="H27" s="5"/>
       <x:c r="I27" s="5" t="s">
-        <x:v>499</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="J27" s="7"/>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="11" t="s">
-        <x:v>500</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B28" s="13">
         <x:v>45367</x:v>
@@ -5995,19 +6013,19 @@
         <x:v>济州汉拿山</x:v>
       </x:c>
       <x:c r="E28" s="5" t="s">
-        <x:v>501</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="F28" s="5"/>
       <x:c r="G28" s="5"/>
       <x:c r="H28" s="5"/>
       <x:c r="I28" s="5" t="s">
-        <x:v>502</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="J28" s="7"/>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="11" t="s">
-        <x:v>503</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B29" s="13">
         <x:v>45315</x:v>
@@ -6019,19 +6037,19 @@
         <x:v>茂朱滑雪</x:v>
       </x:c>
       <x:c r="E29" s="5" t="s">
-        <x:v>504</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="F29" s="5"/>
       <x:c r="G29" s="5"/>
       <x:c r="H29" s="5"/>
       <x:c r="I29" s="5" t="s">
-        <x:v>505</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="J29" s="7"/>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="11" t="s">
-        <x:v>506</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B30" s="13">
         <x:v>45276</x:v>
@@ -6043,19 +6061,19 @@
         <x:v>我和雪人</x:v>
       </x:c>
       <x:c r="E30" s="5" t="s">
-        <x:v>507</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="F30" s="5"/>
       <x:c r="G30" s="5"/>
       <x:c r="H30" s="5"/>
       <x:c r="I30" s="5" t="s">
-        <x:v>508</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="J30" s="7"/>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="11" t="s">
-        <x:v>509</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="B31" s="13">
         <x:v>45218</x:v>
@@ -6067,19 +6085,19 @@
         <x:v>波兰卡托维兹μTAS</x:v>
       </x:c>
       <x:c r="E31" s="5" t="s">
-        <x:v>510</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="F31" s="5"/>
       <x:c r="G31" s="5"/>
       <x:c r="H31" s="5"/>
       <x:c r="I31" s="5" t="s">
-        <x:v>511</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="J31" s="7"/>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="11" t="s">
-        <x:v>512</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="B32" s="13">
         <x:v>45161</x:v>
@@ -6091,19 +6109,19 @@
         <x:v>釜山广安里</x:v>
       </x:c>
       <x:c r="E32" s="5" t="s">
-        <x:v>513</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="F32" s="5"/>
       <x:c r="G32" s="5"/>
       <x:c r="H32" s="5"/>
       <x:c r="I32" s="5" t="s">
-        <x:v>514</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="J32" s="7"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="11" t="s">
-        <x:v>515</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="B33" s="13">
         <x:v>45137</x:v>
@@ -6115,19 +6133,19 @@
         <x:v>济州牛岛</x:v>
       </x:c>
       <x:c r="E33" s="5" t="s">
-        <x:v>516</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="F33" s="5"/>
       <x:c r="G33" s="5"/>
       <x:c r="H33" s="5"/>
       <x:c r="I33" s="5" t="s">
-        <x:v>517</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="J33" s="7"/>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="11" t="s">
-        <x:v>518</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B34" s="13">
         <x:v>45059</x:v>
@@ -6139,19 +6157,19 @@
         <x:v>Dr. Dongsu 婚礼</x:v>
       </x:c>
       <x:c r="E34" s="5" t="s">
-        <x:v>519</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="F34" s="5"/>
       <x:c r="G34" s="5"/>
       <x:c r="H34" s="5"/>
       <x:c r="I34" s="5" t="s">
-        <x:v>520</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="J34" s="7"/>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="11" t="s">
-        <x:v>521</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="B35" s="13">
         <x:v>44947</x:v>
@@ -6163,19 +6181,19 @@
         <x:v>韩国过年</x:v>
       </x:c>
       <x:c r="E35" s="5" t="s">
-        <x:v>522</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="F35" s="5"/>
       <x:c r="G35" s="5"/>
       <x:c r="H35" s="5"/>
       <x:c r="I35" s="5" t="s">
-        <x:v>523</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="J35" s="7"/>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="11" t="s">
-        <x:v>524</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="B36" s="13">
         <x:v>44884</x:v>
@@ -6187,19 +6205,19 @@
         <x:v>光州无等山</x:v>
       </x:c>
       <x:c r="E36" s="5" t="s">
-        <x:v>525</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="F36" s="5"/>
       <x:c r="G36" s="5"/>
       <x:c r="H36" s="5"/>
       <x:c r="I36" s="5" t="s">
-        <x:v>526</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="J36" s="7"/>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="11" t="s">
-        <x:v>527</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="B37" s="13">
         <x:v>44805</x:v>
@@ -6211,13 +6229,13 @@
         <x:v>抵达韩国</x:v>
       </x:c>
       <x:c r="E37" s="5" t="s">
-        <x:v>528</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="F37" s="5"/>
       <x:c r="G37" s="5"/>
       <x:c r="H37" s="5"/>
       <x:c r="I37" s="5" t="s">
-        <x:v>529</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="J37" s="7"/>
     </x:row>
@@ -6364,6 +6382,30 @@
         <x:v>20260912_SATURN 演出.jpg</x:v>
       </x:c>
       <x:c r="J43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>gallery_043</x:v>
+      </x:c>
+      <x:c r="B44" s="17" t="n">
+        <x:v>46290</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>60 km Mid-Autumn Festival Ride</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>中秋骑行60km</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>assets/albums-optimized/20260925_%E4%B8%AD%E7%A7%8B%E9%AA%91%E8%A1%8C60km.webp</x:v>
+      </x:c>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+      <x:c r="I44" t="str">
+        <x:v>20260925_中秋骑行60km.jpg</x:v>
+      </x:c>
+      <x:c r="J44"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -6373,7 +6415,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f58cfe67e604e87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R423adc9f23974451"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6394,13 +6436,13 @@
   <x:sheetData>
     <x:row r="1" ht="27.950000762939453" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>530</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B1" s="9" t="s">
-        <x:v>531</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>532</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
         <x:v>36</x:v>
@@ -6418,7 +6460,7 @@
         <x:v>294</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>377</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="J1" s="3" t="s">
         <x:v>3</x:v>
@@ -6426,17 +6468,17 @@
     </x:row>
     <x:row r="2" ht="63.95000076293945" customHeight="1">
       <x:c r="A2" s="4" t="s">
-        <x:v>533</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="B2" s="10" t="s">
-        <x:v>534</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="C2" s="4"/>
       <x:c r="D2" s="4" t="s">
-        <x:v>535</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
-        <x:v>536</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4" t="s">
@@ -6452,19 +6494,19 @@
     </x:row>
     <x:row r="3" ht="63.95000076293945" customHeight="1">
       <x:c r="A3" s="5" t="s">
+        <x:v>533</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="s">
+        <x:v>534</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="s">
+        <x:v>535</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="s">
+        <x:v>536</x:v>
+      </x:c>
+      <x:c r="E3" s="5" t="s">
         <x:v>537</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="s">
-        <x:v>538</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="s">
-        <x:v>539</x:v>
-      </x:c>
-      <x:c r="D3" s="5" t="s">
-        <x:v>540</x:v>
-      </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>541</x:v>
       </x:c>
       <x:c r="F3" s="5"/>
       <x:c r="G3" s="5"/>
@@ -6476,19 +6518,19 @@
     </x:row>
     <x:row r="4" ht="63.95000076293945" customHeight="1">
       <x:c r="A4" s="5" t="s">
-        <x:v>537</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="B4" s="11" t="s">
-        <x:v>542</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>543</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>544</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>545</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="F4" s="5"/>
       <x:c r="G4" s="5"/>
@@ -6500,24 +6542,24 @@
     </x:row>
     <x:row r="5" ht="63.95000076293945" customHeight="1">
       <x:c r="A5" s="5" t="s">
-        <x:v>546</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B5" s="11" t="s">
-        <x:v>547</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="C5" s="5"/>
       <x:c r="D5" s="5" t="s">
-        <x:v>548</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>549</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5" t="s">
-        <x:v>550</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="H5" s="5" t="s">
-        <x:v>551</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="I5" s="5">
         <x:v>1</x:v>
@@ -6526,24 +6568,24 @@
     </x:row>
     <x:row r="6" ht="63.95000076293945" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>546</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B6" s="11" t="s">
-        <x:v>552</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="C6" s="5"/>
       <x:c r="D6" s="5" t="s">
-        <x:v>553</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>554</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5" t="s">
-        <x:v>555</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="H6" s="5" t="s">
-        <x:v>556</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="I6" s="5">
         <x:v>2</x:v>
@@ -6552,24 +6594,24 @@
     </x:row>
     <x:row r="7" ht="63.95000076293945" customHeight="1">
       <x:c r="A7" s="5" t="s">
-        <x:v>546</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B7" s="11" t="s">
-        <x:v>557</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="C7" s="5"/>
       <x:c r="D7" s="5" t="s">
-        <x:v>558</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>559</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="F7" s="5"/>
       <x:c r="G7" s="5" t="s">
-        <x:v>560</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="H7" s="5" t="s">
-        <x:v>561</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="I7" s="5">
         <x:v>3</x:v>
@@ -6578,24 +6620,24 @@
     </x:row>
     <x:row r="8" ht="63.95000076293945" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>546</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B8" s="11" t="s">
-        <x:v>562</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="C8" s="5"/>
       <x:c r="D8" s="5" t="s">
-        <x:v>563</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>564</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="F8" s="5"/>
       <x:c r="G8" s="5" t="s">
-        <x:v>565</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="H8" s="5" t="s">
-        <x:v>566</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="I8" s="5">
         <x:v>4</x:v>
@@ -6604,24 +6646,24 @@
     </x:row>
     <x:row r="9" ht="63.95000076293945" customHeight="1">
       <x:c r="A9" s="5" t="s">
-        <x:v>546</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B9" s="11" t="s">
-        <x:v>567</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="C9" s="5"/>
       <x:c r="D9" s="5" t="s">
-        <x:v>568</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>569</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="F9" s="5"/>
       <x:c r="G9" s="5" t="s">
-        <x:v>570</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="H9" s="5" t="s">
-        <x:v>571</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="I9" s="5">
         <x:v>5</x:v>
@@ -6630,24 +6672,24 @@
     </x:row>
     <x:row r="10" ht="63.95000076293945" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>572</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="B10" s="11" t="s">
-        <x:v>573</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="C10" s="5"/>
       <x:c r="D10" s="5" t="s">
-        <x:v>574</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>575</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="F10" s="5"/>
       <x:c r="G10" s="5" t="s">
-        <x:v>576</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="H10" s="5" t="s">
-        <x:v>577</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="I10" s="5">
         <x:v>1</x:v>
@@ -6656,24 +6698,24 @@
     </x:row>
     <x:row r="11" ht="63.95000076293945" customHeight="1">
       <x:c r="A11" s="5" t="s">
-        <x:v>572</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="B11" s="11" t="s">
-        <x:v>578</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="C11" s="5"/>
       <x:c r="D11" s="5" t="s">
-        <x:v>579</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>580</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="F11" s="5"/>
       <x:c r="G11" s="5" t="s">
-        <x:v>581</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="H11" s="5" t="s">
-        <x:v>582</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="I11" s="5">
         <x:v>2</x:v>
@@ -6682,24 +6724,24 @@
     </x:row>
     <x:row r="12" ht="63.95000076293945" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>572</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="B12" s="11" t="s">
-        <x:v>583</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="C12" s="5"/>
       <x:c r="D12" s="5" t="s">
-        <x:v>584</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>585</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="F12" s="5"/>
       <x:c r="G12" s="5" t="s">
-        <x:v>586</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="H12" s="5" t="s">
-        <x:v>587</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="I12" s="5">
         <x:v>3</x:v>
@@ -6708,24 +6750,24 @@
     </x:row>
     <x:row r="13" ht="63.95000076293945" customHeight="1">
       <x:c r="A13" s="5" t="s">
-        <x:v>572</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="B13" s="11" t="s">
-        <x:v>588</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="C13" s="5"/>
       <x:c r="D13" s="5" t="s">
-        <x:v>589</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>590</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="F13" s="5"/>
       <x:c r="G13" s="5" t="s">
-        <x:v>591</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="H13" s="5" t="s">
-        <x:v>592</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="I13" s="5">
         <x:v>4</x:v>
@@ -6734,24 +6776,24 @@
     </x:row>
     <x:row r="14" ht="63.95000076293945" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>572</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="B14" s="11" t="s">
-        <x:v>593</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="C14" s="5"/>
       <x:c r="D14" s="5" t="s">
-        <x:v>594</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>595</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="F14" s="5"/>
       <x:c r="G14" s="5" t="s">
-        <x:v>596</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="H14" s="5" t="s">
-        <x:v>597</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="I14" s="5">
         <x:v>5</x:v>
@@ -6760,109 +6802,109 @@
     </x:row>
     <x:row r="15" ht="63.95000076293945" customHeight="1">
       <x:c r="A15" s="5" t="s">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="s">
+        <x:v>595</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="s">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="s">
+        <x:v>596</x:v>
+      </x:c>
+      <x:c r="E15" s="5" t="s">
+        <x:v>597</x:v>
+      </x:c>
+      <x:c r="F15" s="5" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="G15" s="5" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="B15" s="11" t="s">
+      <x:c r="H15" s="5" t="s">
         <x:v>599</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>381</x:v>
-      </x:c>
-      <x:c r="D15" s="5" t="s">
-        <x:v>600</x:v>
-      </x:c>
-      <x:c r="E15" s="5" t="s">
-        <x:v>601</x:v>
-      </x:c>
-      <x:c r="F15" s="5" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="G15" s="5" t="s">
-        <x:v>602</x:v>
-      </x:c>
-      <x:c r="H15" s="5" t="s">
-        <x:v>603</x:v>
       </x:c>
       <x:c r="I15" s="5">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J15" s="7" t="s">
-        <x:v>604</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="63.95000076293945" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>598</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="B16" s="11" t="s">
+        <x:v>601</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="E16" s="5" t="s">
+        <x:v>603</x:v>
+      </x:c>
+      <x:c r="F16" s="5" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="G16" s="5" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="H16" s="5" t="s">
         <x:v>605</x:v>
-      </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="D16" s="5" t="s">
-        <x:v>606</x:v>
-      </x:c>
-      <x:c r="E16" s="5" t="s">
-        <x:v>607</x:v>
-      </x:c>
-      <x:c r="F16" s="5" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="G16" s="5" t="s">
-        <x:v>608</x:v>
-      </x:c>
-      <x:c r="H16" s="5" t="s">
-        <x:v>609</x:v>
       </x:c>
       <x:c r="I16" s="5">
         <x:v>2</x:v>
       </x:c>
       <x:c r="J16" s="7" t="s">
-        <x:v>610</x:v>
+        <x:v>606</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="63.95000076293945" customHeight="1">
       <x:c r="A17" s="5" t="s">
-        <x:v>598</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="B17" s="11" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="C17" s="5" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="D17" s="5" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="E17" s="5" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="F17" s="5" t="s">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="G17" s="5" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="H17" s="5" t="s">
         <x:v>611</x:v>
-      </x:c>
-      <x:c r="C17" s="5" t="s">
-        <x:v>410</x:v>
-      </x:c>
-      <x:c r="D17" s="5" t="s">
-        <x:v>612</x:v>
-      </x:c>
-      <x:c r="E17" s="5" t="s">
-        <x:v>613</x:v>
-      </x:c>
-      <x:c r="F17" s="5" t="s">
-        <x:v>382</x:v>
-      </x:c>
-      <x:c r="G17" s="5" t="s">
-        <x:v>614</x:v>
-      </x:c>
-      <x:c r="H17" s="5" t="s">
-        <x:v>615</x:v>
       </x:c>
       <x:c r="I17" s="5">
         <x:v>3</x:v>
       </x:c>
       <x:c r="J17" s="7" t="s">
-        <x:v>616</x:v>
+        <x:v>612</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="63.95000076293945" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>617</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B18" s="11" t="s">
-        <x:v>618</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>619</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
         <x:v>49</x:v>
@@ -6874,10 +6916,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="G18" s="5" t="s">
-        <x:v>620</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="H18" s="5" t="s">
-        <x:v>620</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="I18" s="5">
         <x:v>1</x:v>
@@ -6886,13 +6928,13 @@
     </x:row>
     <x:row r="19" ht="63.95000076293945" customHeight="1">
       <x:c r="A19" s="5" t="s">
+        <x:v>613</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="s">
         <x:v>617</x:v>
       </x:c>
-      <x:c r="B19" s="11" t="s">
-        <x:v>621</x:v>
-      </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D19" s="5" t="s">
         <x:v>60</x:v>
@@ -6904,10 +6946,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
-        <x:v>623</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="H19" s="5" t="s">
-        <x:v>623</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="I19" s="5">
         <x:v>2</x:v>
@@ -6916,13 +6958,13 @@
     </x:row>
     <x:row r="20" ht="63.95000076293945" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>617</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B20" s="11" t="s">
-        <x:v>624</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D20" s="5" t="s">
         <x:v>68</x:v>
@@ -6934,10 +6976,10 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
-        <x:v>625</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="H20" s="5" t="s">
-        <x:v>625</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="I20" s="5">
         <x:v>3</x:v>
@@ -6946,13 +6988,13 @@
     </x:row>
     <x:row r="21" ht="63.95000076293945" customHeight="1">
       <x:c r="A21" s="5" t="s">
-        <x:v>617</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B21" s="11" t="s">
-        <x:v>626</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="C21" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D21" s="5" t="s">
         <x:v>93</x:v>
@@ -6964,10 +7006,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="G21" s="5" t="s">
-        <x:v>627</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="H21" s="5" t="s">
-        <x:v>627</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="I21" s="5">
         <x:v>4</x:v>
@@ -6976,13 +7018,13 @@
     </x:row>
     <x:row r="22" ht="63.95000076293945" customHeight="1">
       <x:c r="A22" s="5" t="s">
-        <x:v>617</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B22" s="11" t="s">
-        <x:v>628</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>629</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
         <x:v>110</x:v>
@@ -6994,10 +7036,10 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="G22" s="5" t="s">
-        <x:v>630</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="H22" s="5" t="s">
-        <x:v>630</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="I22" s="5">
         <x:v>5</x:v>
@@ -7006,13 +7048,13 @@
     </x:row>
     <x:row r="23" ht="63.95000076293945" customHeight="1">
       <x:c r="A23" s="5" t="s">
-        <x:v>631</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B23" s="11" t="s">
-        <x:v>632</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
-        <x:v>619</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="D23" s="5" t="s">
         <x:v>238</x:v>
@@ -7021,13 +7063,13 @@
         <x:v>238</x:v>
       </x:c>
       <x:c r="F23" s="5" t="s">
-        <x:v>633</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="G23" s="5" t="s">
-        <x:v>634</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="H23" s="5" t="s">
-        <x:v>634</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="I23" s="5">
         <x:v>1</x:v>
@@ -7036,13 +7078,13 @@
     </x:row>
     <x:row r="24" ht="63.95000076293945" customHeight="1">
       <x:c r="A24" s="5" t="s">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="s">
         <x:v>631</x:v>
       </x:c>
-      <x:c r="B24" s="11" t="s">
-        <x:v>635</x:v>
-      </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D24" s="5" t="s">
         <x:v>244</x:v>
@@ -7051,13 +7093,13 @@
         <x:v>244</x:v>
       </x:c>
       <x:c r="F24" s="5" t="s">
-        <x:v>636</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="G24" s="5" t="s">
-        <x:v>637</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="H24" s="5" t="s">
-        <x:v>637</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="I24" s="5">
         <x:v>2</x:v>
@@ -7066,13 +7108,13 @@
     </x:row>
     <x:row r="25" ht="63.95000076293945" customHeight="1">
       <x:c r="A25" s="5" t="s">
-        <x:v>631</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B25" s="11" t="s">
-        <x:v>638</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="C25" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D25" s="5" t="s">
         <x:v>272</x:v>
@@ -7081,13 +7123,13 @@
         <x:v>272</x:v>
       </x:c>
       <x:c r="F25" s="5" t="s">
-        <x:v>639</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="G25" s="5" t="s">
-        <x:v>640</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="H25" s="5" t="s">
-        <x:v>640</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="I25" s="5">
         <x:v>3</x:v>
@@ -7096,13 +7138,13 @@
     </x:row>
     <x:row r="26" ht="63.95000076293945" customHeight="1">
       <x:c r="A26" s="5" t="s">
-        <x:v>631</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B26" s="11" t="s">
-        <x:v>641</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D26" s="5" t="s">
         <x:v>282</x:v>
@@ -7111,13 +7153,13 @@
         <x:v>282</x:v>
       </x:c>
       <x:c r="F26" s="5" t="s">
-        <x:v>642</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="G26" s="5" t="s">
-        <x:v>643</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="H26" s="5" t="s">
-        <x:v>643</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="I26" s="5">
         <x:v>4</x:v>
@@ -7126,13 +7168,13 @@
     </x:row>
     <x:row r="27" ht="63.95000076293945" customHeight="1">
       <x:c r="A27" s="5" t="s">
-        <x:v>631</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B27" s="11" t="s">
-        <x:v>644</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="C27" s="5" t="s">
-        <x:v>629</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D27" s="5" t="s">
         <x:v>255</x:v>
@@ -7141,13 +7183,13 @@
         <x:v>255</x:v>
       </x:c>
       <x:c r="F27" s="5" t="s">
-        <x:v>645</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="G27" s="5" t="s">
-        <x:v>646</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="H27" s="5" t="s">
-        <x:v>646</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="I27" s="5">
         <x:v>5</x:v>
@@ -7156,24 +7198,24 @@
     </x:row>
     <x:row r="28" ht="63.95000076293945" customHeight="1">
       <x:c r="A28" s="5" t="s">
-        <x:v>647</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="B28" s="11" t="s">
-        <x:v>648</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="C28" s="5"/>
       <x:c r="D28" s="5" t="s">
-        <x:v>649</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="E28" s="5" t="s">
-        <x:v>650</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="F28" s="5"/>
       <x:c r="G28" s="5" t="s">
-        <x:v>651</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="H28" s="5" t="s">
-        <x:v>652</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="I28" s="5">
         <x:v>1</x:v>
@@ -7182,10 +7224,10 @@
     </x:row>
     <x:row r="29" ht="63.95000076293945" customHeight="1">
       <x:c r="A29" s="5" t="s">
-        <x:v>647</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="B29" s="11" t="s">
-        <x:v>653</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="C29" s="5"/>
       <x:c r="D29" s="5" t="s">
@@ -7196,10 +7238,10 @@
       </x:c>
       <x:c r="F29" s="5"/>
       <x:c r="G29" s="5" t="s">
-        <x:v>654</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="H29" s="5" t="s">
-        <x:v>655</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="I29" s="5">
         <x:v>2</x:v>
@@ -7208,10 +7250,10 @@
     </x:row>
     <x:row r="30" ht="63.95000076293945" customHeight="1">
       <x:c r="A30" s="5" t="s">
-        <x:v>647</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="B30" s="11" t="s">
-        <x:v>656</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="C30" s="5"/>
       <x:c r="D30" s="5" t="s">
@@ -7222,10 +7264,10 @@
       </x:c>
       <x:c r="F30" s="5"/>
       <x:c r="G30" s="5" t="s">
-        <x:v>657</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="H30" s="5" t="s">
-        <x:v>658</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="I30" s="5">
         <x:v>3</x:v>
@@ -7234,10 +7276,10 @@
     </x:row>
     <x:row r="31" ht="63.95000076293945" customHeight="1">
       <x:c r="A31" s="5" t="s">
-        <x:v>647</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="B31" s="11" t="s">
-        <x:v>659</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="C31" s="5"/>
       <x:c r="D31" s="5" t="s">
@@ -7248,10 +7290,10 @@
       </x:c>
       <x:c r="F31" s="5"/>
       <x:c r="G31" s="5" t="s">
-        <x:v>660</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="H31" s="5" t="s">
-        <x:v>661</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="I31" s="5">
         <x:v>4</x:v>
@@ -7260,10 +7302,10 @@
     </x:row>
     <x:row r="32" ht="63.95000076293945" customHeight="1">
       <x:c r="A32" s="5" t="s">
-        <x:v>647</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="B32" s="11" t="s">
-        <x:v>662</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="C32" s="5"/>
       <x:c r="D32" s="5" t="s">
@@ -7274,10 +7316,10 @@
       </x:c>
       <x:c r="F32" s="5"/>
       <x:c r="G32" s="5" t="s">
-        <x:v>663</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="H32" s="5" t="s">
-        <x:v>664</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="I32" s="5">
         <x:v>5</x:v>
@@ -7286,13 +7328,13 @@
     </x:row>
     <x:row r="33" ht="63.95000076293945" customHeight="1">
       <x:c r="A33" s="5" t="s">
-        <x:v>665</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="B33" s="11" t="s">
-        <x:v>666</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="C33" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D33" s="5" t="s">
         <x:v>296</x:v>
@@ -7302,10 +7344,10 @@
       </x:c>
       <x:c r="F33" s="5"/>
       <x:c r="G33" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="H33" s="5" t="s">
-        <x:v>667</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="I33" s="5">
         <x:v>1</x:v>
@@ -7314,13 +7356,13 @@
     </x:row>
     <x:row r="34" ht="63.95000076293945" customHeight="1">
       <x:c r="A34" s="5" t="s">
-        <x:v>665</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="B34" s="11" t="s">
-        <x:v>668</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="C34" s="5" t="s">
-        <x:v>622</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="D34" s="5" t="s">
         <x:v>316</x:v>
@@ -7330,10 +7372,10 @@
       </x:c>
       <x:c r="F34" s="5"/>
       <x:c r="G34" s="5" t="s">
-        <x:v>669</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="H34" s="5" t="s">
-        <x:v>669</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="I34" s="5">
         <x:v>2</x:v>
@@ -7342,13 +7384,13 @@
     </x:row>
     <x:row r="35" ht="63.95000076293945" customHeight="1">
       <x:c r="A35" s="5" t="s">
-        <x:v>665</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="B35" s="11" t="s">
-        <x:v>670</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="C35" s="5" t="s">
-        <x:v>671</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="D35" s="5" t="s">
         <x:v>302</x:v>
@@ -7358,10 +7400,10 @@
       </x:c>
       <x:c r="F35" s="5"/>
       <x:c r="G35" s="5" t="s">
-        <x:v>672</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="H35" s="5" t="s">
-        <x:v>672</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="I35" s="5">
         <x:v>3</x:v>
@@ -7370,13 +7412,13 @@
     </x:row>
     <x:row r="36" ht="63.95000076293945" customHeight="1">
       <x:c r="A36" s="5" t="s">
-        <x:v>665</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="B36" s="11" t="s">
-        <x:v>673</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="C36" s="5" t="s">
-        <x:v>674</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="D36" s="5" t="s">
         <x:v>309</x:v>
@@ -7386,10 +7428,10 @@
       </x:c>
       <x:c r="F36" s="5"/>
       <x:c r="G36" s="5" t="s">
-        <x:v>675</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="H36" s="5" t="s">
-        <x:v>675</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="I36" s="5">
         <x:v>4</x:v>
@@ -7399,7 +7441,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2bf5b5d9fca49b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42f1628d5b414870"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7421,19 +7463,19 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>676</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>677</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>678</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
         <x:v>45</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
-        <x:v>376</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="G1" s="3" t="s">
         <x:v>3</x:v>
@@ -7444,13 +7486,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B2" s="4" t="s">
-        <x:v>679</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="C2" s="4" t="s">
-        <x:v>680</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="D2" s="4" t="s">
-        <x:v>681</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="E2" s="4" t="s">
         <x:v>16</x:v>
@@ -7459,7 +7501,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="G2" s="6" t="s">
-        <x:v>682</x:v>
+        <x:v>678</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -7467,16 +7509,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>683</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>684</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="D3" s="5" t="s">
         <x:v>20</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F3" s="5" t="s">
         <x:v>57</x:v>
@@ -7485,19 +7527,19 @@
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="11" t="s">
-        <x:v>685</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>686</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>686</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>687</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F4" s="5" t="s">
         <x:v>57</x:v>
@@ -7506,19 +7548,19 @@
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>688</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>689</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>689</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>690</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F5" s="5" t="s">
         <x:v>57</x:v>
@@ -7527,19 +7569,19 @@
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>691</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>382</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>692</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>693</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>366</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="F6" s="5" t="s">
         <x:v>57</x:v>
@@ -7548,133 +7590,133 @@
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>694</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>695</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>695</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D7" s="5"/>
       <x:c r="E7" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F7" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
       <x:c r="G7" s="7" t="s">
-        <x:v>696</x:v>
+        <x:v>692</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>697</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>698</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>698</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D8" s="5"/>
       <x:c r="E8" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F8" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
       <x:c r="G8" s="7" t="s">
-        <x:v>696</x:v>
+        <x:v>692</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>699</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>700</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="C9" s="5"/>
       <x:c r="D9" s="5" t="s">
-        <x:v>701</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>702</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="F9" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>703</x:v>
+        <x:v>699</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>704</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>705</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="C10" s="5"/>
       <x:c r="D10" s="5" t="s">
-        <x:v>706</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>702</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="F10" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>703</x:v>
+        <x:v>699</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>707</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="B11" s="5"/>
       <x:c r="C11" s="5" t="s">
-        <x:v>708</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>709</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>702</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="F11" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>710</x:v>
+        <x:v>706</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>711</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="B12" s="5"/>
       <x:c r="C12" s="5" t="s">
-        <x:v>712</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>713</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>702</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="F12" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="G12" s="7" t="s">
-        <x:v>710</x:v>
+        <x:v>706</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="11" t="s">
-        <x:v>714</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
         <x:v>49</x:v>
@@ -7686,7 +7728,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F13" s="5" t="s">
         <x:v>57</x:v>
@@ -7695,7 +7737,7 @@
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="11" t="s">
-        <x:v>716</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
         <x:v>60</x:v>
@@ -7707,7 +7749,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
         <x:v>57</x:v>
@@ -7716,7 +7758,7 @@
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="11" t="s">
-        <x:v>717</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
         <x:v>68</x:v>
@@ -7728,7 +7770,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F15" s="5" t="s">
         <x:v>57</x:v>
@@ -7737,7 +7779,7 @@
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>718</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
         <x:v>77</x:v>
@@ -7749,7 +7791,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
         <x:v>57</x:v>
@@ -7758,7 +7800,7 @@
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="11" t="s">
-        <x:v>719</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
         <x:v>86</x:v>
@@ -7770,7 +7812,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F17" s="5" t="s">
         <x:v>57</x:v>
@@ -7779,7 +7821,7 @@
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>720</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
         <x:v>93</x:v>
@@ -7791,7 +7833,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F18" s="5" t="s">
         <x:v>57</x:v>
@@ -7800,7 +7842,7 @@
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="11" t="s">
-        <x:v>721</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
         <x:v>103</x:v>
@@ -7812,7 +7854,7 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="E19" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F19" s="5" t="s">
         <x:v>57</x:v>
@@ -7821,7 +7863,7 @@
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="11" t="s">
-        <x:v>722</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
         <x:v>110</x:v>
@@ -7833,7 +7875,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F20" s="5" t="s">
         <x:v>57</x:v>
@@ -7842,7 +7884,7 @@
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="11" t="s">
-        <x:v>723</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="B21" s="5" t="s">
         <x:v>119</x:v>
@@ -7854,7 +7896,7 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="E21" s="5" t="s">
-        <x:v>715</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="F21" s="5" t="s">
         <x:v>57</x:v>
@@ -7863,7 +7905,7 @@
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="11" t="s">
-        <x:v>724</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
         <x:v>238</x:v>
@@ -7884,7 +7926,7 @@
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="11" t="s">
-        <x:v>725</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
         <x:v>244</x:v>
@@ -7905,7 +7947,7 @@
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="11" t="s">
-        <x:v>726</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
         <x:v>255</x:v>
@@ -7926,7 +7968,7 @@
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="11" t="s">
-        <x:v>727</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="B25" s="5" t="s">
         <x:v>272</x:v>
@@ -7947,7 +7989,7 @@
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="11" t="s">
-        <x:v>728</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
         <x:v>278</x:v>
@@ -7977,7 +8019,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e3101ca1cd340b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R207b488c0b794746"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
content: update publications and gallery
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Radbd3e8e219948e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="Rdd80c23f3ec34e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="Rbd2b160797b54d36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R275538baa40549e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R0e9b6e0a1982471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="Rff96d16248634970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R896606a52cd744c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R9a696770eb1f41b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="Rd0a326455d314de1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rdf160f993c7641e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R153ea13ea4794031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R0bbc2c19f5aa46f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R91c05f6c9d154181"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R73e2e4a9daed45ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R1c5db975f2204b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R0e0dfcb62dd54982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R6ca1e9669abf44b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="Rd81379b83f924a4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2473,8 +2473,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="publicationsTable" displayName="publicationsTable" ref="A1:O13" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:O13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="publicationsTable" displayName="publicationsTable" ref="A1:O14" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:O14"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="year"/>
@@ -2583,8 +2583,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J44" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:J44"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J46" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J46"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="date"/>
@@ -2977,7 +2977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77aba52755e94f36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55a73af4a46c404f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3579,6 +3579,57 @@
         <x:v>Published online: 2026-07-30. Online ahead of print. PMID: 42528395.</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>pub_013</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>A Self-Coupling Microcantilever-Probe Platform: Non-compressive Sustained Assessment of Cardiac Contractility and Cardiotoxicity Screening</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>A Self-Coupling Microcantilever-Probe Platform: Non-compressive Sustained Assessment of Cardiac Contractility and Cardiotoxicity Screening</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Haolan Sun, Longlong Li, Eung-Sam Kim, Bong-Kee Lee, Dong-Weon Lee</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Sensors and Actuators Reports</x:v>
+      </x:c>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14" t="str">
+        <x:v>100516</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>10.1016/j.snr.2026.100516</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/pii/S2666053926000834</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>journal</x:v>
+      </x:c>
+      <x:c r="M14" s="15" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>@article{sun2026selfcoupling,
+  title = {A Self-Coupling Microcantilever-Probe Platform: Non-compressive Sustained Assessment of Cardiac Contractility and Cardiotoxicity Screening},
+  author = {Haolan Sun and Longlong Li and Eung-Sam Kim and Bong-Kee Lee and Dong-Weon Lee},
+  journal = {Sensors and Actuators Reports},
+  year = {2026},
+  pages = {100516},
+  doi = {10.1016/j.snr.2026.100516},
+  url = {https://www.sciencedirect.com/science/article/pii/S2666053926000834}
+}</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>Published online: 2026-09-30. ISSN: 2666-0539. Volume and issue were not yet assigned in the verified publisher record.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="L2:L10">
@@ -3590,7 +3641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc47d3b7dddc84c08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra93ff4bec4f7439a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4245,7 +4296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0cef20cf2b462f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01de866bf96649b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4651,7 +4702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8eb1f759cb194c04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92762a3e137f4bfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5085,7 +5136,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1f1eb5179214f77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0cca217d4f4ceb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5324,7 +5375,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e9903a50edc455f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66dfc8cd92fe4d07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6407,6 +6458,54 @@
       </x:c>
       <x:c r="J44"/>
     </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>gallery_044</x:v>
+      </x:c>
+      <x:c r="B45" s="17" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>MNTL at Gyeongju World</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>MNTL+庆州世界</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>assets/albums-optimized/20260930_MNTL%2B%E5%BA%86%E5%B7%9E%E4%B8%96%E7%95%8C.webp</x:v>
+      </x:c>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+      <x:c r="I45" t="str">
+        <x:v>20260930_MNTL+庆州世界.jpg</x:v>
+      </x:c>
+      <x:c r="J45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>gallery_045</x:v>
+      </x:c>
+      <x:c r="B46" s="17" t="n">
+        <x:v>46297</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>I ♥ MNTL: Off-Road Riding in Gyeongju</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>I♥MNTL+庆州越野</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>assets/albums-optimized/20261002_I%E2%99%A5MNTL%2B%E5%BA%86%E5%B7%9E%E8%B6%8A%E9%87%8E.webp</x:v>
+      </x:c>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46" t="str">
+        <x:v>20261002_I♥MNTL+庆州越野.jpg</x:v>
+      </x:c>
+      <x:c r="J46"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F2:F37">
@@ -6415,7 +6514,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R423adc9f23974451"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R037bdde3f4464c99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7441,7 +7540,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42f1628d5b414870"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R765ffa7e591a487c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8019,7 +8118,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R207b488c0b794746"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raefcc639d74a4f96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
content: add Gangneung fishing gallery photo
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rdf160f993c7641e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R153ea13ea4794031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R0bbc2c19f5aa46f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R91c05f6c9d154181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R73e2e4a9daed45ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R1c5db975f2204b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R0e0dfcb62dd54982"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R6ca1e9669abf44b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="Rd81379b83f924a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="R22e058c0361b4767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R8ae7bc6d297b4c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R062475b3ea97401d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R160907d84d4649e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R45dfb35ba6e94ebb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="Rc05c2e230f284b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R34fc7a1e6e314eaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R6e1eb99875c64df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R7bebd6fee3724689"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2583,8 +2583,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J46" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:J46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J47" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J47"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="date"/>
@@ -2977,7 +2977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55a73af4a46c404f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R483e46639f144242"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3641,7 +3641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra93ff4bec4f7439a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra843fc6ad2a54a8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4296,7 +4296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01de866bf96649b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64166ea838eb4ea2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4702,7 +4702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92762a3e137f4bfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb20c3cd08c9d477c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5136,7 +5136,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa0cca217d4f4ceb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radfcc96352864294"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5375,7 +5375,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66dfc8cd92fe4d07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5b717c261694893"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6506,6 +6506,30 @@
       </x:c>
       <x:c r="J46"/>
     </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>gallery_046</x:v>
+      </x:c>
+      <x:c r="B47" s="17" t="d">
+        <x:v>2026-10-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>Deep-Sea Fishing for a Giant Catch in Gangneung</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>江陵出海钓深海巨物</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>assets/albums-optimized/20261009_%E6%B1%9F%E9%99%B5%E5%87%BA%E6%B5%B7%E9%92%93%E6%B7%B1%E6%B5%B7%E5%B7%A8%E7%89%A9.webp</x:v>
+      </x:c>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47" t="str">
+        <x:v>20261009_江陵出海钓深海巨物.jpg</x:v>
+      </x:c>
+      <x:c r="J47"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F2:F37">
@@ -6514,7 +6538,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R037bdde3f4464c99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58e9b995a64a4a5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7540,7 +7564,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R765ffa7e591a487c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9b3cbeaece427a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8118,7 +8142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raefcc639d74a4f96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda286ceee3e44fa9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
content: add IEEE-NANOMED gallery entry
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="R22e058c0361b4767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R8ae7bc6d297b4c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R062475b3ea97401d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R160907d84d4649e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R45dfb35ba6e94ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="Rc05c2e230f284b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R34fc7a1e6e314eaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="R6e1eb99875c64df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R7bebd6fee3724689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rd30fd3dcaf524eea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R42c657c4ee51444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="Rc37a5f76ef664fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R29663772a1af4254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R8a43fc6839534600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R7cdc283399d4411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R22dedb8bb2b14947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="Rd414c246e10d4a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="Rfee75f5a6c4d440e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2583,8 +2583,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J47" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:J47"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="galleryTable" displayName="galleryTable" ref="A1:J48" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:J48"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="date"/>
@@ -2977,7 +2977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R483e46639f144242"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cbab228f3d745a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3641,7 +3641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra843fc6ad2a54a8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8297c63f78f44baf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4296,7 +4296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64166ea838eb4ea2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0b1ec5e26aa4db4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4702,7 +4702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb20c3cd08c9d477c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf090e805dc6046c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5136,7 +5136,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radfcc96352864294"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e050445cfb4acc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5375,7 +5375,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5b717c261694893"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0069ade285e4792"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6530,6 +6530,30 @@
       </x:c>
       <x:c r="J47"/>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>gallery_047</x:v>
+      </x:c>
+      <x:c r="B48" s="17" t="d">
+        <x:v>2024-12-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Online Oral Presentation at IEEE-NANOMED 2024 (Best Paper Session)</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>在NanoMed进行在线口头发表（Best Paper Session）</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>assets/albums-optimized/20241204_NanoMed%E5%9C%A8%E7%BA%BF%E5%8F%A3%E5%A4%B4%E5%8F%91%E8%A1%A8_BestPaperSession.webp</x:v>
+      </x:c>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+      <x:c r="I48" t="str">
+        <x:v>20241204_NanoMed在线口头发表_BestPaperSession.png</x:v>
+      </x:c>
+      <x:c r="J48"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="F2:F37">
@@ -6538,7 +6562,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58e9b995a64a4a5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3fa96ce0164978"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7564,7 +7588,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9b3cbeaece427a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab6d42a7494f4a27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8142,7 +8166,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda286ceee3e44fa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c8c88106cfe4457"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
content: add LinkedIn profile link
</commit_message>
<xml_diff>
--- a/data/website_content.xlsx
+++ b/data/website_content.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="Rd30fd3dcaf524eea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="R42c657c4ee51444d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="Rc37a5f76ef664fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R29663772a1af4254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R8a43fc6839534600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R7cdc283399d4411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R22dedb8bb2b14947"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="Rd414c246e10d4a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="Rfee75f5a6c4d440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="profile" sheetId="1" r:id="R927b2cea066b48ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="publications" sheetId="2" r:id="Rec68bc60545f4381"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patents" sheetId="3" r:id="R118fd9d7dc9746d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conferences" sheetId="4" r:id="R0dc28af33d0542dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="awards" sheetId="5" r:id="R04c1f7edf5964f84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="6" r:id="R4e4c71c73b074b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery" sheetId="7" r:id="R08653bf3c94b4c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cv" sheetId="8" r:id="Re4ca863405094099"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="links" sheetId="9" r:id="R41bbb759e79e4658"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,8 +2621,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="linksTable" displayName="linksTable" ref="A1:G26">
-  <x:autoFilter ref="A1:G26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="linksTable" displayName="linksTable" ref="A1:G27" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:G27"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="label_en"/>
@@ -2977,7 +2977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cbab228f3d745a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reacfba51eec04f13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3641,7 +3641,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8297c63f78f44baf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb15b780588ed4727"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4296,7 +4296,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0b1ec5e26aa4db4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb15d1d7094f466b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4702,7 +4702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf090e805dc6046c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R073ccb3388924554"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5136,7 +5136,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e050445cfb4acc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9399b4998fd440a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5375,7 +5375,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0069ade285e4792"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88301a2969354c69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6562,7 +6562,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3fa96ce0164978"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b23865dbbd4e2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7588,7 +7588,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab6d42a7494f4a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72c18e4a97da4f4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8155,6 +8155,27 @@
       </x:c>
       <x:c r="G26" s="7"/>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>linkedin</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>LinkedIn</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>LinkedIn</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>https://www.linkedin.com/in/longlong-li-11a7123a2/</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>profile</x:v>
+      </x:c>
+      <x:c r="F27" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G27"/>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="E2:E26">
@@ -8166,7 +8187,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c8c88106cfe4457"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd0d6ad63ee24b4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>